<commit_message>
pipeline test buy SPY 2026-10-06T20:00Z
</commit_message>
<xml_diff>
--- a/fund_state/live/ledger/fund_positions.xlsx
+++ b/fund_state/live/ledger/fund_positions.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="K2" s="4" t="n"/>
       <c r="L2" s="4" t="n">
-        <v>1045.970092773438</v>
+        <v>1028.359985351562</v>
       </c>
       <c r="M2" s="5">
         <f>IFERROR(IF(E2="Short",-1,1)*(IF(K2&lt;&gt;"",K2,L2)/J2-1),"")</f>
@@ -685,7 +685,7 @@
       </c>
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="n">
-        <v>1066.170043945312</v>
+        <v>1045.885009765625</v>
       </c>
       <c r="M3" s="5">
         <f>IFERROR(IF(E3="Short",-1,1)*(IF(K3&lt;&gt;"",K3,L3)/J3-1),"")</f>
@@ -754,7 +754,7 @@
       </c>
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="n">
-        <v>67.83000183105469</v>
+        <v>68.71499633789062</v>
       </c>
       <c r="M4" s="5">
         <f>IFERROR(IF(E4="Short",-1,1)*(IF(K4&lt;&gt;"",K4,L4)/J4-1),"")</f>
@@ -823,7 +823,7 @@
       </c>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n">
-        <v>506.5599975585938</v>
+        <v>505.8800048828125</v>
       </c>
       <c r="M5" s="5">
         <f>IFERROR(IF(E5="Short",-1,1)*(IF(K5&lt;&gt;"",K5,L5)/J5-1),"")</f>
@@ -892,7 +892,7 @@
       </c>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="n">
-        <v>94.09100341796875</v>
+        <v>93.56999969482422</v>
       </c>
       <c r="M6" s="5">
         <f>IFERROR(IF(E6="Short",-1,1)*(IF(K6&lt;&gt;"",K6,L6)/J6-1),"")</f>
@@ -961,7 +961,7 @@
       </c>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n">
-        <v>115.2249984741211</v>
+        <v>116.3199996948242</v>
       </c>
       <c r="M7" s="5">
         <f>IFERROR(IF(E7="Short",-1,1)*(IF(K7&lt;&gt;"",K7,L7)/J7-1),"")</f>

</xml_diff>

<commit_message>
pipeline test sell SPY 2026-10-07T20:00Z
</commit_message>
<xml_diff>
--- a/fund_state/live/ledger/fund_positions.xlsx
+++ b/fund_state/live/ledger/fund_positions.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Positions'!$A$1:$Q$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Orders'!$A$1:$O$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Positions'!$A$1:$Q$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Orders'!$A$1:$O$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Account'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cash activity'!$A$1:$F$3</definedName>
   </definedNames>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -579,22 +579,22 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>SPDR S&amp;P 500 ETF</t>
+          <t>GE Vernova</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>beta hedge</t>
+          <t>position</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Short</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -604,19 +604,19 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="3" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>777.52001953125</v>
+        <v>987.38</v>
       </c>
       <c r="K2" s="4" t="n"/>
       <c r="L2" s="4" t="n">
-        <v>777.530029296875</v>
+        <v>997.5800170898438</v>
       </c>
       <c r="M2" s="5">
         <f>IFERROR(IF(E2="Short",-1,1)*(IF(K2&lt;&gt;"",K2,L2)/J2-1),"")</f>
@@ -626,11 +626,17 @@
         <f>IFERROR(I2*(IF(K2&lt;&gt;"",K2,L2)-J2),"")</f>
         <v/>
       </c>
-      <c r="O2" s="7" t="n"/>
-      <c r="P2" s="2" t="n"/>
+      <c r="O2" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>uphold</t>
+        </is>
+      </c>
       <c r="Q2" s="8" t="inlineStr">
         <is>
-          <t>SPY hedge to zero beta</t>
+          <t>NRC construction permit for GEV/Hitachi's new reactor design (Sep 29-30) is a concrete regulatory milestone that validates the nuclear growth story, whose coverage share jumped to 49% from 9%. With no earnings next week and only 1.1% gain last week, the news is not fully priced; GLJ's Sell is opinion, not information.</t>
         </is>
       </c>
     </row>
@@ -642,12 +648,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>GE Vernova</t>
+          <t>Micron Technology</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -675,11 +681,11 @@
         <v>2</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>987.38</v>
+        <v>1097.61</v>
       </c>
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="n">
-        <v>997.7000122070312</v>
+        <v>1087.630004882812</v>
       </c>
       <c r="M3" s="5">
         <f>IFERROR(IF(E3="Short",-1,1)*(IF(K3&lt;&gt;"",K3,L3)/J3-1),"")</f>
@@ -694,12 +700,12 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>uphold</t>
+          <t>weaken</t>
         </is>
       </c>
       <c r="Q3" s="8" t="inlineStr">
         <is>
-          <t>NRC construction permit for GEV/Hitachi's new reactor design (Sep 29-30) is a concrete regulatory milestone that validates the nuclear growth story, whose coverage share jumped to 49% from 9%. With no earnings next week and only 1.1% gain last week, the news is not fully priced; GLJ's Sell is opinion, not information.</t>
+          <t>Micron's Sep 30 Q4 beat with above-Street guidance on AI memory demand confirms the bull case, and the AI memory rally story's coverage share is rising (37% vs 29% avg) with a new AI Memory Boom narrative accelerating. Post-earnings drift should favor MU next week, though Burry's puts and bubble fears cap conviction.</t>
         </is>
       </c>
     </row>
@@ -711,12 +717,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -731,7 +737,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Closed (daily review)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -739,22 +745,16 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
+      <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="3" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>1097.61</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>1087.910034179688</v>
-      </c>
+        <v>67.84999999999999</v>
+      </c>
+      <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="n">
-        <v>1087.780029296875</v>
+        <v>69.70500183105469</v>
       </c>
       <c r="M4" s="5">
         <f>IFERROR(IF(E4="Short",-1,1)*(IF(K4&lt;&gt;"",K4,L4)/J4-1),"")</f>
@@ -765,16 +765,16 @@
         <v/>
       </c>
       <c r="O4" s="7" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>weaken</t>
+          <t>uphold</t>
         </is>
       </c>
       <c r="Q4" s="8" t="inlineStr">
         <is>
-          <t>Micron's Sep 30 Q4 beat with above-Street guidance on AI memory demand confirms the bull case, and the AI memory rally story's coverage share is rising (37% vs 29% avg) with a new AI Memory Boom narrative accelerating. Post-earnings drift should favor MU next week, though Burry's puts and bubble fears cap conviction.</t>
+          <t>Deutsche Bank's Sep 29 upgrade to Buy is a new story now 40% of coverage, and the selloff-debate narrative is fading, suggesting a near-term bounce. But the upgrade came with a lowered target and weak engagement trends persist, capping conviction.</t>
         </is>
       </c>
     </row>
@@ -786,12 +786,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>BRK.B</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>Berkshire Hathaway</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Short</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -811,19 +811,19 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="3" t="n">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>1087.910034179688</v>
+        <v>500.56</v>
       </c>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n">
-        <v>1087.780029296875</v>
+        <v>506.2950134277344</v>
       </c>
       <c r="M5" s="5">
         <f>IFERROR(IF(E5="Short",-1,1)*(IF(K5&lt;&gt;"",K5,L5)/J5-1),"")</f>
@@ -838,12 +838,12 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>weaken</t>
+          <t>uphold</t>
         </is>
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>Micron's Sep 30 Q4 beat with above-Street guidance on AI memory demand confirms the bull case, and the AI memory rally story's coverage share is rising (37% vs 29% avg) with a new AI Memory Boom narrative accelerating. Post-earnings drift should favor MU next week, though Burry's puts and bubble fears cap conviction.</t>
+          <t>Buffett's chairman exit and Howard's appointment add governance uncertainty, while the positive Abel/Alphabet narrative fades. Lennar stake increase is too small to offset. Expect slight underperformance next week.</t>
         </is>
       </c>
     </row>
@@ -855,12 +855,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Netflix</t>
+          <t>Lululemon Athletica</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Short</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -885,14 +885,14 @@
       </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="3" t="n">
-        <v>24</v>
+        <v>-27</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>67.84999999999999</v>
+        <v>95.87</v>
       </c>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="n">
-        <v>69.69499969482422</v>
+        <v>91.86299896240234</v>
       </c>
       <c r="M6" s="5">
         <f>IFERROR(IF(E6="Short",-1,1)*(IF(K6&lt;&gt;"",K6,L6)/J6-1),"")</f>
@@ -903,7 +903,7 @@
         <v/>
       </c>
       <c r="O6" s="7" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -912,7 +912,7 @@
       </c>
       <c r="Q6" s="8" t="inlineStr">
         <is>
-          <t>Deutsche Bank's Sep 29 upgrade to Buy is a new story now 40% of coverage, and the selloff-debate narrative is fading, suggesting a near-term bounce. But the upgrade came with a lowered target and weak engagement trends persist, capping conviction.</t>
+          <t>Fresh Sep 30 cash-flow skepticism and Sep 25 CEO/bylaw governance changes add to negative sentiment from Sep 3 guidance cut. With no earnings next week, LULU likely underperforms as the market questions cash durability and leadership transition.</t>
         </is>
       </c>
     </row>
@@ -924,12 +924,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>BRK.B</t>
+          <t>STZ</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Berkshire Hathaway</t>
+          <t>Constellation Brands</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -954,14 +954,14 @@
       </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="3" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>500.56</v>
+        <v>112.95</v>
       </c>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n">
-        <v>506.2250061035156</v>
+        <v>118.3199996948242</v>
       </c>
       <c r="M7" s="5">
         <f>IFERROR(IF(E7="Short",-1,1)*(IF(K7&lt;&gt;"",K7,L7)/J7-1),"")</f>
@@ -972,7 +972,7 @@
         <v/>
       </c>
       <c r="O7" s="7" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
@@ -981,156 +981,12 @@
       </c>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>Buffett's chairman exit and Howard's appointment add governance uncertainty, while the positive Abel/Alphabet narrative fades. Lennar stake increase is too small to offset. Expect slight underperformance next week.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>LULU</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Lululemon Athletica</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>position</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Short</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="3" t="n">
-        <v>-27</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>95.87</v>
-      </c>
-      <c r="K8" s="4" t="n"/>
-      <c r="L8" s="4" t="n">
-        <v>91.88999938964844</v>
-      </c>
-      <c r="M8" s="5">
-        <f>IFERROR(IF(E8="Short",-1,1)*(IF(K8&lt;&gt;"",K8,L8)/J8-1),"")</f>
-        <v/>
-      </c>
-      <c r="N8" s="6">
-        <f>IFERROR(I8*(IF(K8&lt;&gt;"",K8,L8)-J8),"")</f>
-        <v/>
-      </c>
-      <c r="O8" s="7" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>uphold</t>
-        </is>
-      </c>
-      <c r="Q8" s="8" t="inlineStr">
-        <is>
-          <t>Fresh Sep 30 cash-flow skepticism and Sep 25 CEO/bylaw governance changes add to negative sentiment from Sep 3 guidance cut. With no earnings next week, LULU likely underperforms as the market questions cash durability and leadership transition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>STZ</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Constellation Brands</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>position</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Short</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Closed (daily review)</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="n">
-        <v>-5</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>112.95</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>118.3150024414062</v>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>118.3199996948242</v>
-      </c>
-      <c r="M9" s="5">
-        <f>IFERROR(IF(E9="Short",-1,1)*(IF(K9&lt;&gt;"",K9,L9)/J9-1),"")</f>
-        <v/>
-      </c>
-      <c r="N9" s="6">
-        <f>IFERROR(I9*(IF(K9&lt;&gt;"",K9,L9)-J9),"")</f>
-        <v/>
-      </c>
-      <c r="O9" s="7" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>uphold</t>
-        </is>
-      </c>
-      <c r="Q9" s="8" t="inlineStr">
-        <is>
           <t>New earnings story dominates: Q2 on Oct 6 expected EPS decline, negative ESP, and analyst target cuts. Selloff/outlook stories fading, but stock already down 12.8% in a month, so edge is modest. Binary event warrants lower confidence.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q9"/>
+  <autoFilter ref="A1:Q7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1141,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2145,7 +2001,7 @@
       </c>
       <c r="K16" s="4" t="n"/>
       <c r="L16" s="4" t="n">
-        <v>185.009994506836</v>
+        <v>185.0099945068359</v>
       </c>
       <c r="M16" s="10" t="n"/>
       <c r="N16" s="9">
@@ -2462,182 +2318,8 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>MU</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>review-reduce</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>market-on-close (daily review)</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="n">
-        <v>1086.89</v>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>filled</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="n"/>
-      <c r="L22" s="4" t="n"/>
-      <c r="M22" s="10" t="n"/>
-      <c r="N22" s="9">
-        <f>IFERROR(G22*IF(K22&lt;&gt;"",K22,I22),"")</f>
-        <v/>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>fund-2026-09-30-MU-r20261007</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>STZ</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>review-exit</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="G23" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>market-on-close (daily review)</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="n">
-        <v>117.985</v>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>filled</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="n"/>
-      <c r="L23" s="4" t="n"/>
-      <c r="M23" s="10" t="n"/>
-      <c r="N23" s="9">
-        <f>IFERROR(G23*IF(K23&lt;&gt;"",K23,I23),"")</f>
-        <v/>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>fund-2026-09-30-STZ-r20261007</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>review-rehedge</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>market-on-close (daily review)</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="n">
-        <v>777.515</v>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>filled</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="n"/>
-      <c r="L24" s="4" t="n"/>
-      <c r="M24" s="10" t="n"/>
-      <c r="N24" s="9">
-        <f>IFERROR(G24*IF(K24&lt;&gt;"",K24,I24),"")</f>
-        <v/>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>fund-2026-09-30-SPY-r20261007</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O24"/>
+  <autoFilter ref="A1:O21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fund memo + performance 2026-10-07T23:45Z
</commit_message>
<xml_diff>
--- a/fund_state/live/ledger/fund_positions.xlsx
+++ b/fund_state/live/ledger/fund_positions.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Positions'!$A$1:$Q$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Orders'!$A$1:$O$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Positions'!$A$1:$Q$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Orders'!$A$1:$O$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Account'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cash activity'!$A$1:$F$3</definedName>
   </definedNames>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -612,11 +612,11 @@
         <v>-1</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>777.260009765625</v>
+        <v>777.219970703125</v>
       </c>
       <c r="K2" s="4" t="n"/>
       <c r="L2" s="4" t="n">
-        <v>777.260009765625</v>
+        <v>777.219970703125</v>
       </c>
       <c r="M2" s="5">
         <f>IFERROR(IF(E2="Short",-1,1)*(IF(K2&lt;&gt;"",K2,L2)/J2-1),"")</f>
@@ -679,7 +679,7 @@
       </c>
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="n">
-        <v>997.6300048828125</v>
+        <v>997.0900268554688</v>
       </c>
       <c r="M3" s="5">
         <f>IFERROR(IF(E3="Short",-1,1)*(IF(K3&lt;&gt;"",K3,L3)/J3-1),"")</f>
@@ -731,7 +731,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed (daily review)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -739,14 +739,20 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="I4" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>1097.61</v>
       </c>
-      <c r="K4" s="4" t="n"/>
+      <c r="K4" s="4" t="n">
+        <v>1088</v>
+      </c>
       <c r="L4" s="4" t="n">
         <v>1088</v>
       </c>
@@ -780,12 +786,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Netflix</t>
+          <t>Micron Technology</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -805,19 +811,19 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="3" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>67.84999999999999</v>
+        <v>1088</v>
       </c>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n">
-        <v>69.69999694824219</v>
+        <v>1088</v>
       </c>
       <c r="M5" s="5">
         <f>IFERROR(IF(E5="Short",-1,1)*(IF(K5&lt;&gt;"",K5,L5)/J5-1),"")</f>
@@ -828,16 +834,16 @@
         <v/>
       </c>
       <c r="O5" s="7" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>uphold</t>
+          <t>weaken</t>
         </is>
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>Deutsche Bank's Sep 29 upgrade to Buy is a new story now 40% of coverage, and the selloff-debate narrative is fading, suggesting a near-term bounce. But the upgrade came with a lowered target and weak engagement trends persist, capping conviction.</t>
+          <t>Micron's Sep 30 Q4 beat with above-Street guidance on AI memory demand confirms the bull case, and the AI memory rally story's coverage share is rising (37% vs 29% avg) with a new AI Memory Boom narrative accelerating. Post-earnings drift should favor MU next week, though Burry's puts and bubble fears cap conviction.</t>
         </is>
       </c>
     </row>
@@ -849,12 +855,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>BRK.B</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Berkshire Hathaway</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -864,7 +870,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Short</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -879,14 +885,14 @@
       </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="3" t="n">
-        <v>-4</v>
+        <v>24</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>500.56</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="n">
-        <v>506.260009765625</v>
+        <v>69.69999694824219</v>
       </c>
       <c r="M6" s="5">
         <f>IFERROR(IF(E6="Short",-1,1)*(IF(K6&lt;&gt;"",K6,L6)/J6-1),"")</f>
@@ -897,7 +903,7 @@
         <v/>
       </c>
       <c r="O6" s="7" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -906,7 +912,7 @@
       </c>
       <c r="Q6" s="8" t="inlineStr">
         <is>
-          <t>Buffett's chairman exit and Howard's appointment add governance uncertainty, while the positive Abel/Alphabet narrative fades. Lennar stake increase is too small to offset. Expect slight underperformance next week.</t>
+          <t>Deutsche Bank's Sep 29 upgrade to Buy is a new story now 40% of coverage, and the selloff-debate narrative is fading, suggesting a near-term bounce. But the upgrade came with a lowered target and weak engagement trends persist, capping conviction.</t>
         </is>
       </c>
     </row>
@@ -918,12 +924,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>BRK.B</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Lululemon Athletica</t>
+          <t>Berkshire Hathaway</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -948,14 +954,14 @@
       </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="3" t="n">
-        <v>-27</v>
+        <v>-4</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>95.87</v>
+        <v>500.56</v>
       </c>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n">
-        <v>91.87999725341797</v>
+        <v>506.25</v>
       </c>
       <c r="M7" s="5">
         <f>IFERROR(IF(E7="Short",-1,1)*(IF(K7&lt;&gt;"",K7,L7)/J7-1),"")</f>
@@ -975,7 +981,7 @@
       </c>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>Fresh Sep 30 cash-flow skepticism and Sep 25 CEO/bylaw governance changes add to negative sentiment from Sep 3 guidance cut. With no earnings next week, LULU likely underperforms as the market questions cash durability and leadership transition.</t>
+          <t>Buffett's chairman exit and Howard's appointment add governance uncertainty, while the positive Abel/Alphabet narrative fades. Lennar stake increase is too small to offset. Expect slight underperformance next week.</t>
         </is>
       </c>
     </row>
@@ -987,12 +993,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>STZ</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Constellation Brands</t>
+          <t>Lululemon Athletica</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1007,7 +1013,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Closed (daily review)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1015,22 +1021,16 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
+      <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="3" t="n">
-        <v>-5</v>
+        <v>-27</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>112.95</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>118.3899993896484</v>
-      </c>
+        <v>95.87</v>
+      </c>
+      <c r="K8" s="4" t="n"/>
       <c r="L8" s="4" t="n">
-        <v>118.3899993896484</v>
+        <v>91.87999725341797</v>
       </c>
       <c r="M8" s="5">
         <f>IFERROR(IF(E8="Short",-1,1)*(IF(K8&lt;&gt;"",K8,L8)/J8-1),"")</f>
@@ -1041,21 +1041,96 @@
         <v/>
       </c>
       <c r="O8" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>uphold</t>
+        </is>
+      </c>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>Fresh Sep 30 cash-flow skepticism and Sep 25 CEO/bylaw governance changes add to negative sentiment from Sep 3 guidance cut. With no earnings next week, LULU likely underperforms as the market questions cash durability and leadership transition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>STZ</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Constellation Brands</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Closed (daily review)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>-5</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>112.95</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>118.3899993896484</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>118.3899993896484</v>
+      </c>
+      <c r="M9" s="5">
+        <f>IFERROR(IF(E9="Short",-1,1)*(IF(K9&lt;&gt;"",K9,L9)/J9-1),"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="6">
+        <f>IFERROR(I9*(IF(K9&lt;&gt;"",K9,L9)-J9),"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="7" t="n">
         <v>0.55</v>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>uphold</t>
         </is>
       </c>
-      <c r="Q8" s="8" t="inlineStr">
+      <c r="Q9" s="8" t="inlineStr">
         <is>
           <t>New earnings story dominates: Q2 on Oct 6 expected EPS decline, negative ESP, and analyst target cuts. Selloff/outlook stories fading, but stock already down 12.8% in a month, so edge is modest. Binary event warrants lower confidence.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q8"/>
+  <autoFilter ref="A1:Q9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1066,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2400,24 +2475,24 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>STZ</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>review-exit</t>
+          <t>review-reduce</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="F22" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -2425,7 +2500,7 @@
         </is>
       </c>
       <c r="I22" s="4" t="n">
-        <v>117.985</v>
+        <v>1086.89</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
@@ -2441,7 +2516,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>fund-2026-09-30-STZ-r20261007</t>
+          <t>fund-2026-09-30-MU-r20261007</t>
         </is>
       </c>
     </row>
@@ -2458,24 +2533,24 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>STZ</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>review-rehedge</t>
+          <t>review-exit</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="F23" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -2483,7 +2558,7 @@
         </is>
       </c>
       <c r="I23" s="4" t="n">
-        <v>777.515</v>
+        <v>117.985</v>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
@@ -2499,12 +2574,70 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
+          <t>fund-2026-09-30-STZ-r20261007</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>review-rehedge</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>market-on-close (daily review)</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>777.515</v>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="n"/>
+      <c r="L24" s="4" t="n"/>
+      <c r="M24" s="10" t="n"/>
+      <c r="N24" s="9">
+        <f>IFERROR(G24*IF(K24&lt;&gt;"",K24,I24),"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
           <t>fund-2026-09-30-SPY-r20261007</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O23"/>
+  <autoFilter ref="A1:O24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fund memo + performance 2026-10-08T07:59Z
</commit_message>
<xml_diff>
--- a/fund_state/live/ledger/fund_positions.xlsx
+++ b/fund_state/live/ledger/fund_positions.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="K2" s="4" t="n"/>
       <c r="L2" s="4" t="n">
-        <v>779.0900268554688</v>
+        <v>777.219970703125</v>
       </c>
       <c r="M2" s="5">
         <f>IFERROR(IF(E2="Short",-1,1)*(IF(K2&lt;&gt;"",K2,L2)/J2-1),"")</f>
@@ -679,7 +679,7 @@
       </c>
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="n">
-        <v>1029.2099609375</v>
+        <v>997.0900268554688</v>
       </c>
       <c r="M3" s="5">
         <f>IFERROR(IF(E3="Short",-1,1)*(IF(K3&lt;&gt;"",K3,L3)/J3-1),"")</f>
@@ -731,7 +731,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed (daily review)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -739,16 +739,22 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="I4" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>1097.61</v>
       </c>
-      <c r="K4" s="4" t="n"/>
+      <c r="K4" s="4" t="n">
+        <v>1086.75</v>
+      </c>
       <c r="L4" s="4" t="n">
-        <v>1045.56005859375</v>
+        <v>1088</v>
       </c>
       <c r="M4" s="5">
         <f>IFERROR(IF(E4="Short",-1,1)*(IF(K4&lt;&gt;"",K4,L4)/J4-1),"")</f>
@@ -817,7 +823,7 @@
       </c>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n">
-        <v>1045.56005859375</v>
+        <v>1088</v>
       </c>
       <c r="M5" s="5">
         <f>IFERROR(IF(E5="Short",-1,1)*(IF(K5&lt;&gt;"",K5,L5)/J5-1),"")</f>
@@ -886,7 +892,7 @@
       </c>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="n">
-        <v>68.69000244140625</v>
+        <v>69.69999694824219</v>
       </c>
       <c r="M6" s="5">
         <f>IFERROR(IF(E6="Short",-1,1)*(IF(K6&lt;&gt;"",K6,L6)/J6-1),"")</f>
@@ -955,7 +961,7 @@
       </c>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n">
-        <v>505.5400085449219</v>
+        <v>506.25</v>
       </c>
       <c r="M7" s="5">
         <f>IFERROR(IF(E7="Short",-1,1)*(IF(K7&lt;&gt;"",K7,L7)/J7-1),"")</f>
@@ -1024,7 +1030,7 @@
       </c>
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="4" t="n">
-        <v>93.61000061035156</v>
+        <v>91.87999725341797</v>
       </c>
       <c r="M8" s="5">
         <f>IFERROR(IF(E8="Short",-1,1)*(IF(K8&lt;&gt;"",K8,L8)/J8-1),"")</f>
@@ -1076,7 +1082,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed (daily review)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1084,16 +1090,22 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="I9" s="3" t="n">
         <v>-5</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>112.95</v>
       </c>
-      <c r="K9" s="4" t="n"/>
+      <c r="K9" s="4" t="n">
+        <v>118.22</v>
+      </c>
       <c r="L9" s="4" t="n">
-        <v>115.6699981689453</v>
+        <v>118.3899993896484</v>
       </c>
       <c r="M9" s="5">
         <f>IFERROR(IF(E9="Short",-1,1)*(IF(K9&lt;&gt;"",K9,L9)/J9-1),"")</f>

</xml_diff>

<commit_message>
fund memo + performance 2026-10-14T23:59Z
</commit_message>
<xml_diff>
--- a/fund_state/live/ledger/fund_positions.xlsx
+++ b/fund_state/live/ledger/fund_positions.xlsx
@@ -490,11 +490,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Account value (Alpaca, 2026-10-14 16:15 ET)</t>
+          <t>Account value (Alpaca, 2026-10-14 19:59 ET)</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>98829.89079999999</v>
+        <v>98744.07239999999</v>
       </c>
     </row>
     <row r="3">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>-1082.539199999999</v>
+        <v>-1168.357599999998</v>
       </c>
     </row>
     <row r="7">
@@ -666,7 +666,7 @@
         <v>621.12</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>568.21</v>
+        <v>554.3662</v>
       </c>
       <c r="H2" s="6">
         <f>D2*G2</f>
@@ -709,7 +709,7 @@
         <v>360.345</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>346.12</v>
+        <v>341.8264</v>
       </c>
       <c r="H3" s="6">
         <f>D3*G3</f>
@@ -752,7 +752,7 @@
         <v>187.69</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>184.51</v>
+        <v>183.9695</v>
       </c>
       <c r="H4" s="6">
         <f>D4*G4</f>
@@ -795,7 +795,7 @@
         <v>500.56</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>526.3</v>
+        <v>527.248</v>
       </c>
       <c r="H5" s="6">
         <f>D5*G5</f>
@@ -838,7 +838,7 @@
         <v>285.07</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>279.92</v>
+        <v>276.25</v>
       </c>
       <c r="H6" s="6">
         <f>D6*G6</f>
@@ -881,7 +881,7 @@
         <v>348.4111111111112</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>346.67</v>
+        <v>344.23</v>
       </c>
       <c r="H7" s="6">
         <f>D7*G7</f>
@@ -924,7 +924,7 @@
         <v>70.92</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>63.0155</v>
+        <v>61.5713</v>
       </c>
       <c r="H8" s="6">
         <f>D8*G8</f>
@@ -967,7 +967,7 @@
         <v>1050.046666666667</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>895</v>
+        <v>869.2934</v>
       </c>
       <c r="H9" s="6">
         <f>D9*G9</f>
@@ -1010,7 +1010,7 @@
         <v>1170.25</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>1209.51</v>
+        <v>1214</v>
       </c>
       <c r="H10" s="6">
         <f>D10*G10</f>
@@ -1053,7 +1053,7 @@
         <v>95.37625</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>94.09</v>
+        <v>93.16</v>
       </c>
       <c r="H11" s="6">
         <f>D11*G11</f>
@@ -1096,7 +1096,7 @@
         <v>236.64</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>238.31</v>
+        <v>238.79</v>
       </c>
       <c r="H12" s="6">
         <f>D12*G12</f>
@@ -1139,7 +1139,7 @@
         <v>720.8100000000001</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>737.7916</v>
+        <v>730.3099999999999</v>
       </c>
       <c r="H13" s="6">
         <f>D13*G13</f>
@@ -1182,7 +1182,7 @@
         <v>274.6186956521739</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>245.25</v>
+        <v>239.45</v>
       </c>
       <c r="H14" s="6">
         <f>D14*G14</f>
@@ -1225,7 +1225,7 @@
         <v>34.76117647058824</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>35.1804</v>
+        <v>35.06</v>
       </c>
       <c r="H15" s="6">
         <f>D15*G15</f>
@@ -1268,7 +1268,7 @@
         <v>230.4985714285714</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>221.474</v>
+        <v>217.94</v>
       </c>
       <c r="H16" s="6">
         <f>D16*G16</f>
@@ -1311,7 +1311,7 @@
         <v>128.19</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>129.24</v>
+        <v>129.74</v>
       </c>
       <c r="H17" s="6">
         <f>D17*G17</f>
@@ -1354,7 +1354,7 @@
         <v>1595.61</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1394</v>
+        <v>1357.5</v>
       </c>
       <c r="H18" s="6">
         <f>D18*G18</f>
@@ -1397,7 +1397,7 @@
         <v>773.95</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>769.02</v>
+        <v>767.1569</v>
       </c>
       <c r="H19" s="6">
         <f>D19*G19</f>
@@ -1440,7 +1440,7 @@
         <v>775.35</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>712.832</v>
+        <v>692.0358</v>
       </c>
       <c r="H20" s="6">
         <f>D20*G20</f>
@@ -1483,7 +1483,7 @@
         <v>393.05</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>363.2</v>
+        <v>353.2632</v>
       </c>
       <c r="H21" s="6">
         <f>D21*G21</f>
@@ -2227,7 +2227,7 @@
         <v>773.95</v>
       </c>
       <c r="L2" s="5" t="n">
-        <v>769.34</v>
+        <v>769.5999755859375</v>
       </c>
       <c r="M2" s="7">
         <f>IFERROR(IF(E2="Short",-1,1)*(IF(K2&lt;&gt;"",K2,L2)/J2-1),"")</f>
@@ -2296,7 +2296,7 @@
         <v>998.54</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>941.67</v>
+        <v>941.780029296875</v>
       </c>
       <c r="M3" s="7">
         <f>IFERROR(IF(E3="Short",-1,1)*(IF(K3&lt;&gt;"",K3,L3)/J3-1),"")</f>
@@ -2371,7 +2371,7 @@
         <v>1086.75</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>912.6799999999999</v>
+        <v>914.1300048828125</v>
       </c>
       <c r="M4" s="7">
         <f>IFERROR(IF(E4="Short",-1,1)*(IF(K4&lt;&gt;"",K4,L4)/J4-1),"")</f>
@@ -2446,7 +2446,7 @@
         <v>1036.16</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>912.6799999999999</v>
+        <v>914.1300048828125</v>
       </c>
       <c r="M5" s="7">
         <f>IFERROR(IF(E5="Short",-1,1)*(IF(K5&lt;&gt;"",K5,L5)/J5-1),"")</f>
@@ -2521,7 +2521,7 @@
         <v>71.59</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>70.58</v>
+        <v>70.56999969482422</v>
       </c>
       <c r="M6" s="7">
         <f>IFERROR(IF(E6="Short",-1,1)*(IF(K6&lt;&gt;"",K6,L6)/J6-1),"")</f>
@@ -2596,7 +2596,7 @@
         <v>511.0499877929688</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>526.5549999999999</v>
+        <v>526.3499755859375</v>
       </c>
       <c r="M7" s="7">
         <f>IFERROR(IF(E7="Short",-1,1)*(IF(K7&lt;&gt;"",K7,L7)/J7-1),"")</f>
@@ -2671,7 +2671,7 @@
         <v>92.70999999999999</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>94.06</v>
+        <v>94.08999633789062</v>
       </c>
       <c r="M8" s="7">
         <f>IFERROR(IF(E8="Short",-1,1)*(IF(K8&lt;&gt;"",K8,L8)/J8-1),"")</f>
@@ -2746,7 +2746,7 @@
         <v>118.22</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>127.46</v>
+        <v>127.4100036621094</v>
       </c>
       <c r="M9" s="7">
         <f>IFERROR(IF(E9="Short",-1,1)*(IF(K9&lt;&gt;"",K9,L9)/J9-1),"")</f>
@@ -2821,7 +2821,7 @@
         <v>778.28</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>769.34</v>
+        <v>769.5999755859375</v>
       </c>
       <c r="M10" s="7">
         <f>IFERROR(IF(E10="Short",-1,1)*(IF(K10&lt;&gt;"",K10,L10)/J10-1),"")</f>
@@ -2890,7 +2890,7 @@
         <v>777.915</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>769.34</v>
+        <v>769.5999755859375</v>
       </c>
       <c r="M11" s="7">
         <f>IFERROR(IF(E11="Short",-1,1)*(IF(K11&lt;&gt;"",K11,L11)/J11-1),"")</f>
@@ -2959,7 +2959,7 @@
         <v>769.5999755859375</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>769.34</v>
+        <v>769.5999755859375</v>
       </c>
       <c r="M12" s="7">
         <f>IFERROR(IF(E12="Short",-1,1)*(IF(K12&lt;&gt;"",K12,L12)/J12-1),"")</f>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="5" t="n">
-        <v>769.34</v>
+        <v>769.5999755859375</v>
       </c>
       <c r="M13" s="7">
         <f>IFERROR(IF(E13="Short",-1,1)*(IF(K13&lt;&gt;"",K13,L13)/J13-1),"")</f>
@@ -3091,7 +3091,7 @@
         <v>605.795</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>570.96</v>
+        <v>570.8200073242188</v>
       </c>
       <c r="M14" s="7">
         <f>IFERROR(IF(E14="Short",-1,1)*(IF(K14&lt;&gt;"",K14,L14)/J14-1),"")</f>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="5" t="n">
-        <v>570.96</v>
+        <v>570.8200073242188</v>
       </c>
       <c r="M15" s="7">
         <f>IFERROR(IF(E15="Short",-1,1)*(IF(K15&lt;&gt;"",K15,L15)/J15-1),"")</f>
@@ -3235,7 +3235,7 @@
         <v>361.53</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>346.34</v>
+        <v>346.25</v>
       </c>
       <c r="M16" s="7">
         <f>IFERROR(IF(E16="Short",-1,1)*(IF(K16&lt;&gt;"",K16,L16)/J16-1),"")</f>
@@ -3310,7 +3310,7 @@
         <v>357.595</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>346.34</v>
+        <v>346.25</v>
       </c>
       <c r="M17" s="7">
         <f>IFERROR(IF(E17="Short",-1,1)*(IF(K17&lt;&gt;"",K17,L17)/J17-1),"")</f>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="5" t="n">
-        <v>346.34</v>
+        <v>346.25</v>
       </c>
       <c r="M18" s="7">
         <f>IFERROR(IF(E18="Short",-1,1)*(IF(K18&lt;&gt;"",K18,L18)/J18-1),"")</f>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="5" t="n">
-        <v>184.58</v>
+        <v>184.6600036621094</v>
       </c>
       <c r="M19" s="7">
         <f>IFERROR(IF(E19="Short",-1,1)*(IF(K19&lt;&gt;"",K19,L19)/J19-1),"")</f>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="5" t="n">
-        <v>279.66</v>
+        <v>279.5400085449219</v>
       </c>
       <c r="M20" s="7">
         <f>IFERROR(IF(E20="Short",-1,1)*(IF(K20&lt;&gt;"",K20,L20)/J20-1),"")</f>
@@ -3586,7 +3586,7 @@
       </c>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="5" t="n">
-        <v>347.78</v>
+        <v>347.6400146484375</v>
       </c>
       <c r="M21" s="7">
         <f>IFERROR(IF(E21="Short",-1,1)*(IF(K21&lt;&gt;"",K21,L21)/J21-1),"")</f>
@@ -3655,7 +3655,7 @@
       </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="5" t="n">
-        <v>63.175</v>
+        <v>63.11000061035156</v>
       </c>
       <c r="M22" s="7">
         <f>IFERROR(IF(E22="Short",-1,1)*(IF(K22&lt;&gt;"",K22,L22)/J22-1),"")</f>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="K23" s="5" t="n"/>
       <c r="L23" s="5" t="n">
-        <v>896.04</v>
+        <v>896.3300170898438</v>
       </c>
       <c r="M23" s="7">
         <f>IFERROR(IF(E23="Short",-1,1)*(IF(K23&lt;&gt;"",K23,L23)/J23-1),"")</f>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="5" t="n">
-        <v>1210.9</v>
+        <v>1208.739990234375</v>
       </c>
       <c r="M24" s="7">
         <f>IFERROR(IF(E24="Short",-1,1)*(IF(K24&lt;&gt;"",K24,L24)/J24-1),"")</f>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="5" t="n">
-        <v>245.465</v>
+        <v>245.2799987792969</v>
       </c>
       <c r="M25" s="7">
         <f>IFERROR(IF(E25="Short",-1,1)*(IF(K25&lt;&gt;"",K25,L25)/J25-1),"")</f>
@@ -3937,7 +3937,7 @@
         <v>221.3000030517578</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>221.49</v>
+        <v>221.3000030517578</v>
       </c>
       <c r="M26" s="7">
         <f>IFERROR(IF(E26="Short",-1,1)*(IF(K26&lt;&gt;"",K26,L26)/J26-1),"")</f>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="5" t="n">
-        <v>221.49</v>
+        <v>221.3000030517578</v>
       </c>
       <c r="M27" s="7">
         <f>IFERROR(IF(E27="Short",-1,1)*(IF(K27&lt;&gt;"",K27,L27)/J27-1),"")</f>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="5" t="n">
-        <v>526.5549999999999</v>
+        <v>526.3499755859375</v>
       </c>
       <c r="M28" s="7">
         <f>IFERROR(IF(E28="Short",-1,1)*(IF(K28&lt;&gt;"",K28,L28)/J28-1),"")</f>
@@ -4144,7 +4144,7 @@
       </c>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="5" t="n">
-        <v>94.06</v>
+        <v>94.08999633789062</v>
       </c>
       <c r="M29" s="7">
         <f>IFERROR(IF(E29="Short",-1,1)*(IF(K29&lt;&gt;"",K29,L29)/J29-1),"")</f>
@@ -4213,7 +4213,7 @@
       </c>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="5" t="n">
-        <v>238.25</v>
+        <v>238.3099975585938</v>
       </c>
       <c r="M30" s="7">
         <f>IFERROR(IF(E30="Short",-1,1)*(IF(K30&lt;&gt;"",K30,L30)/J30-1),"")</f>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="K31" s="5" t="n"/>
       <c r="L31" s="5" t="n">
-        <v>738.24</v>
+        <v>737.5399780273438</v>
       </c>
       <c r="M31" s="7">
         <f>IFERROR(IF(E31="Short",-1,1)*(IF(K31&lt;&gt;"",K31,L31)/J31-1),"")</f>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="K32" s="5" t="n"/>
       <c r="L32" s="5" t="n">
-        <v>35.32</v>
+        <v>35.29999923706055</v>
       </c>
       <c r="M32" s="7">
         <f>IFERROR(IF(E32="Short",-1,1)*(IF(K32&lt;&gt;"",K32,L32)/J32-1),"")</f>
@@ -4426,7 +4426,7 @@
         <v>125.99375</v>
       </c>
       <c r="L33" s="5" t="n">
-        <v>129.34</v>
+        <v>129.2700042724609</v>
       </c>
       <c r="M33" s="7">
         <f>IFERROR(IF(E33="Short",-1,1)*(IF(K33&lt;&gt;"",K33,L33)/J33-1),"")</f>
@@ -4495,7 +4495,7 @@
       </c>
       <c r="K34" s="5" t="n"/>
       <c r="L34" s="5" t="n">
-        <v>129.34</v>
+        <v>129.2700042724609</v>
       </c>
       <c r="M34" s="7">
         <f>IFERROR(IF(E34="Short",-1,1)*(IF(K34&lt;&gt;"",K34,L34)/J34-1),"")</f>
@@ -4570,7 +4570,7 @@
         <v>1581.73</v>
       </c>
       <c r="L35" s="5" t="n">
-        <v>1395.19</v>
+        <v>1403.339965820312</v>
       </c>
       <c r="M35" s="7">
         <f>IFERROR(IF(E35="Short",-1,1)*(IF(K35&lt;&gt;"",K35,L35)/J35-1),"")</f>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="K36" s="5" t="n"/>
       <c r="L36" s="5" t="n">
-        <v>1395.19</v>
+        <v>1403.339965820312</v>
       </c>
       <c r="M36" s="7">
         <f>IFERROR(IF(E36="Short",-1,1)*(IF(K36&lt;&gt;"",K36,L36)/J36-1),"")</f>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="K37" s="5" t="n"/>
       <c r="L37" s="5" t="n">
-        <v>713.12</v>
+        <v>713.5399780273438</v>
       </c>
       <c r="M37" s="7">
         <f>IFERROR(IF(E37="Short",-1,1)*(IF(K37&lt;&gt;"",K37,L37)/J37-1),"")</f>
@@ -4777,7 +4777,7 @@
       </c>
       <c r="K38" s="5" t="n"/>
       <c r="L38" s="5" t="n">
-        <v>363.04</v>
+        <v>364.1000061035156</v>
       </c>
       <c r="M38" s="7">
         <f>IFERROR(IF(E38="Short",-1,1)*(IF(K38&lt;&gt;"",K38,L38)/J38-1),"")</f>

</xml_diff>

<commit_message>
fund memo + performance 2026-10-21T23:44Z
</commit_message>
<xml_diff>
--- a/fund_state/live/ledger/fund_positions.xlsx
+++ b/fund_state/live/ledger/fund_positions.xlsx
@@ -490,11 +490,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Account value (Alpaca, 2026-10-21 16:16 ET)</t>
+          <t>Account value (Alpaca, 2026-10-21 19:44 ET)</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>98554.0092</v>
+        <v>98307.90000000001</v>
       </c>
     </row>
     <row r="3">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>-1928.190799999998</v>
+        <v>-2174.299999999997</v>
       </c>
     </row>
     <row r="7">
@@ -666,7 +666,7 @@
         <v>582.0666666666667</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>551.98</v>
+        <v>541.85</v>
       </c>
       <c r="H2" s="6">
         <f>D2*G2</f>
@@ -709,7 +709,7 @@
         <v>51.19367647058824</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>50.81</v>
+        <v>50.69</v>
       </c>
       <c r="H3" s="6">
         <f>D3*G3</f>
@@ -752,7 +752,7 @@
         <v>245.0494444444445</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>243.8794</v>
+        <v>242</v>
       </c>
       <c r="H4" s="6">
         <f>D4*G4</f>
@@ -795,7 +795,7 @@
         <v>75.45893617021277</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>77.67</v>
+        <v>77.48999999999999</v>
       </c>
       <c r="H5" s="6">
         <f>D5*G5</f>
@@ -838,7 +838,7 @@
         <v>65.19323076923077</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>58.2671</v>
+        <v>57.25</v>
       </c>
       <c r="H6" s="6">
         <f>D6*G6</f>
@@ -881,7 +881,7 @@
         <v>335.42</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>335</v>
+        <v>334.2</v>
       </c>
       <c r="H7" s="6">
         <f>D7*G7</f>
@@ -924,7 +924,7 @@
         <v>23.23999999999999</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>23.45</v>
+        <v>23.5</v>
       </c>
       <c r="H8" s="6">
         <f>D8*G8</f>
@@ -967,7 +967,7 @@
         <v>262.5911428571428</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>243.3839</v>
+        <v>238.77</v>
       </c>
       <c r="H9" s="6">
         <f>D9*G9</f>
@@ -1010,7 +1010,7 @@
         <v>35.49667968750001</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>37.4</v>
+        <v>37.35</v>
       </c>
       <c r="H10" s="6">
         <f>D10*G10</f>
@@ -1053,7 +1053,7 @@
         <v>773.2016666666667</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>773.404</v>
+        <v>769.5599999999999</v>
       </c>
       <c r="H11" s="6">
         <f>D11*G11</f>
@@ -2820,7 +2820,7 @@
         <v>773.95</v>
       </c>
       <c r="L2" s="5" t="n">
-        <v>773.22</v>
+        <v>773.0900268554688</v>
       </c>
       <c r="M2" s="7">
         <f>IFERROR(IF(E2="Short",-1,1)*(IF(K2&lt;&gt;"",K2,L2)/J2-1),"")</f>
@@ -2889,7 +2889,7 @@
         <v>998.54</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>926.21</v>
+        <v>925.9199829101562</v>
       </c>
       <c r="M3" s="7">
         <f>IFERROR(IF(E3="Short",-1,1)*(IF(K3&lt;&gt;"",K3,L3)/J3-1),"")</f>
@@ -2964,7 +2964,7 @@
         <v>1086.75</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>908.08</v>
+        <v>913.6699829101562</v>
       </c>
       <c r="M4" s="7">
         <f>IFERROR(IF(E4="Short",-1,1)*(IF(K4&lt;&gt;"",K4,L4)/J4-1),"")</f>
@@ -3039,7 +3039,7 @@
         <v>1036.16</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>908.08</v>
+        <v>913.6699829101562</v>
       </c>
       <c r="M5" s="7">
         <f>IFERROR(IF(E5="Short",-1,1)*(IF(K5&lt;&gt;"",K5,L5)/J5-1),"")</f>
@@ -3114,7 +3114,7 @@
         <v>71.59</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>65.05</v>
+        <v>65.04000091552734</v>
       </c>
       <c r="M6" s="7">
         <f>IFERROR(IF(E6="Short",-1,1)*(IF(K6&lt;&gt;"",K6,L6)/J6-1),"")</f>
@@ -3189,7 +3189,7 @@
         <v>511.0499877929688</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>540.62</v>
+        <v>538.989990234375</v>
       </c>
       <c r="M7" s="7">
         <f>IFERROR(IF(E7="Short",-1,1)*(IF(K7&lt;&gt;"",K7,L7)/J7-1),"")</f>
@@ -3264,7 +3264,7 @@
         <v>92.70999999999999</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>96.535</v>
+        <v>96.52999877929688</v>
       </c>
       <c r="M8" s="7">
         <f>IFERROR(IF(E8="Short",-1,1)*(IF(K8&lt;&gt;"",K8,L8)/J8-1),"")</f>
@@ -3339,7 +3339,7 @@
         <v>118.22</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>132.03</v>
+        <v>132.0200042724609</v>
       </c>
       <c r="M9" s="7">
         <f>IFERROR(IF(E9="Short",-1,1)*(IF(K9&lt;&gt;"",K9,L9)/J9-1),"")</f>
@@ -3414,7 +3414,7 @@
         <v>778.28</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>773.22</v>
+        <v>773.0900268554688</v>
       </c>
       <c r="M10" s="7">
         <f>IFERROR(IF(E10="Short",-1,1)*(IF(K10&lt;&gt;"",K10,L10)/J10-1),"")</f>
@@ -3483,7 +3483,7 @@
         <v>777.915</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>773.22</v>
+        <v>773.0900268554688</v>
       </c>
       <c r="M11" s="7">
         <f>IFERROR(IF(E11="Short",-1,1)*(IF(K11&lt;&gt;"",K11,L11)/J11-1),"")</f>
@@ -3552,7 +3552,7 @@
         <v>768.885</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>773.22</v>
+        <v>773.0900268554688</v>
       </c>
       <c r="M12" s="7">
         <f>IFERROR(IF(E12="Short",-1,1)*(IF(K12&lt;&gt;"",K12,L12)/J12-1),"")</f>
@@ -3621,7 +3621,7 @@
         <v>771.98</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>773.22</v>
+        <v>773.0900268554688</v>
       </c>
       <c r="M13" s="7">
         <f>IFERROR(IF(E13="Short",-1,1)*(IF(K13&lt;&gt;"",K13,L13)/J13-1),"")</f>
@@ -3690,7 +3690,7 @@
         <v>605.795</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>553.78</v>
+        <v>552.719970703125</v>
       </c>
       <c r="M14" s="7">
         <f>IFERROR(IF(E14="Short",-1,1)*(IF(K14&lt;&gt;"",K14,L14)/J14-1),"")</f>
@@ -3765,7 +3765,7 @@
         <v>562.54</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>553.78</v>
+        <v>552.719970703125</v>
       </c>
       <c r="M15" s="7">
         <f>IFERROR(IF(E15="Short",-1,1)*(IF(K15&lt;&gt;"",K15,L15)/J15-1),"")</f>
@@ -3840,7 +3840,7 @@
         <v>361.53</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>337.87</v>
+        <v>337.7999877929688</v>
       </c>
       <c r="M16" s="7">
         <f>IFERROR(IF(E16="Short",-1,1)*(IF(K16&lt;&gt;"",K16,L16)/J16-1),"")</f>
@@ -3915,7 +3915,7 @@
         <v>357.595</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>337.87</v>
+        <v>337.7999877929688</v>
       </c>
       <c r="M17" s="7">
         <f>IFERROR(IF(E17="Short",-1,1)*(IF(K17&lt;&gt;"",K17,L17)/J17-1),"")</f>
@@ -3990,7 +3990,7 @@
         <v>344.42</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>337.87</v>
+        <v>337.7999877929688</v>
       </c>
       <c r="M18" s="7">
         <f>IFERROR(IF(E18="Short",-1,1)*(IF(K18&lt;&gt;"",K18,L18)/J18-1),"")</f>
@@ -4065,7 +4065,7 @@
         <v>188.498788</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>192.27</v>
+        <v>192.2799987792969</v>
       </c>
       <c r="M19" s="7">
         <f>IFERROR(IF(E19="Short",-1,1)*(IF(K19&lt;&gt;"",K19,L19)/J19-1),"")</f>
@@ -4140,7 +4140,7 @@
         <v>276.52</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>270.63</v>
+        <v>270.739990234375</v>
       </c>
       <c r="M20" s="7">
         <f>IFERROR(IF(E20="Short",-1,1)*(IF(K20&lt;&gt;"",K20,L20)/J20-1),"")</f>
@@ -4215,7 +4215,7 @@
         <v>349.461111</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>334.715</v>
+        <v>334.760009765625</v>
       </c>
       <c r="M21" s="7">
         <f>IFERROR(IF(E21="Short",-1,1)*(IF(K21&lt;&gt;"",K21,L21)/J21-1),"")</f>
@@ -4290,7 +4290,7 @@
         <v>58.7</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>58.17</v>
+        <v>58.16999816894531</v>
       </c>
       <c r="M22" s="7">
         <f>IFERROR(IF(E22="Short",-1,1)*(IF(K22&lt;&gt;"",K22,L22)/J22-1),"")</f>
@@ -4365,7 +4365,7 @@
         <v>869.4233330000001</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>851.22</v>
+        <v>850.7000122070312</v>
       </c>
       <c r="M23" s="7">
         <f>IFERROR(IF(E23="Short",-1,1)*(IF(K23&lt;&gt;"",K23,L23)/J23-1),"")</f>
@@ -4440,7 +4440,7 @@
         <v>1253.68</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>1270.89</v>
+        <v>1270.75</v>
       </c>
       <c r="M24" s="7">
         <f>IFERROR(IF(E24="Short",-1,1)*(IF(K24&lt;&gt;"",K24,L24)/J24-1),"")</f>
@@ -4515,7 +4515,7 @@
         <v>241.535</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>244.66</v>
+        <v>244.7599945068359</v>
       </c>
       <c r="M25" s="7">
         <f>IFERROR(IF(E25="Short",-1,1)*(IF(K25&lt;&gt;"",K25,L25)/J25-1),"")</f>
@@ -4590,7 +4590,7 @@
         <v>221.17</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>221.9</v>
+        <v>221.9700012207031</v>
       </c>
       <c r="M26" s="7">
         <f>IFERROR(IF(E26="Short",-1,1)*(IF(K26&lt;&gt;"",K26,L26)/J26-1),"")</f>
@@ -4665,7 +4665,7 @@
         <v>217.33</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>221.9</v>
+        <v>221.9700012207031</v>
       </c>
       <c r="M27" s="7">
         <f>IFERROR(IF(E27="Short",-1,1)*(IF(K27&lt;&gt;"",K27,L27)/J27-1),"")</f>
@@ -4740,7 +4740,7 @@
         <v>526.15</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>540.62</v>
+        <v>538.989990234375</v>
       </c>
       <c r="M28" s="7">
         <f>IFERROR(IF(E28="Short",-1,1)*(IF(K28&lt;&gt;"",K28,L28)/J28-1),"")</f>
@@ -4815,7 +4815,7 @@
         <v>99.13124999999999</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>96.535</v>
+        <v>96.52999877929688</v>
       </c>
       <c r="M29" s="7">
         <f>IFERROR(IF(E29="Short",-1,1)*(IF(K29&lt;&gt;"",K29,L29)/J29-1),"")</f>
@@ -4890,7 +4890,7 @@
         <v>242.642308</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>246.245</v>
+        <v>246.25</v>
       </c>
       <c r="M30" s="7">
         <f>IFERROR(IF(E30="Short",-1,1)*(IF(K30&lt;&gt;"",K30,L30)/J30-1),"")</f>
@@ -4965,7 +4965,7 @@
         <v>736.4924999999999</v>
       </c>
       <c r="L31" s="5" t="n">
-        <v>718.9400000000001</v>
+        <v>697.52001953125</v>
       </c>
       <c r="M31" s="7">
         <f>IFERROR(IF(E31="Short",-1,1)*(IF(K31&lt;&gt;"",K31,L31)/J31-1),"")</f>
@@ -5040,7 +5040,7 @@
         <v>37.13999938964844</v>
       </c>
       <c r="L32" s="5" t="n">
-        <v>37.525</v>
+        <v>37.52999877929688</v>
       </c>
       <c r="M32" s="7">
         <f>IFERROR(IF(E32="Short",-1,1)*(IF(K32&lt;&gt;"",K32,L32)/J32-1),"")</f>
@@ -5115,7 +5115,7 @@
         <v>125.99375</v>
       </c>
       <c r="L33" s="5" t="n">
-        <v>134.69</v>
+        <v>134.6999969482422</v>
       </c>
       <c r="M33" s="7">
         <f>IFERROR(IF(E33="Short",-1,1)*(IF(K33&lt;&gt;"",K33,L33)/J33-1),"")</f>
@@ -5190,7 +5190,7 @@
         <v>128.4175</v>
       </c>
       <c r="L34" s="5" t="n">
-        <v>134.69</v>
+        <v>134.6999969482422</v>
       </c>
       <c r="M34" s="7">
         <f>IFERROR(IF(E34="Short",-1,1)*(IF(K34&lt;&gt;"",K34,L34)/J34-1),"")</f>
@@ -5265,7 +5265,7 @@
         <v>1581.73</v>
       </c>
       <c r="L35" s="5" t="n">
-        <v>1379.57</v>
+        <v>1378.219970703125</v>
       </c>
       <c r="M35" s="7">
         <f>IFERROR(IF(E35="Short",-1,1)*(IF(K35&lt;&gt;"",K35,L35)/J35-1),"")</f>
@@ -5340,7 +5340,7 @@
         <v>1395.31</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>1379.57</v>
+        <v>1378.219970703125</v>
       </c>
       <c r="M36" s="7">
         <f>IFERROR(IF(E36="Short",-1,1)*(IF(K36&lt;&gt;"",K36,L36)/J36-1),"")</f>
@@ -5415,7 +5415,7 @@
         <v>691.4699999999999</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>697.38</v>
+        <v>696.8900146484375</v>
       </c>
       <c r="M37" s="7">
         <f>IFERROR(IF(E37="Short",-1,1)*(IF(K37&lt;&gt;"",K37,L37)/J37-1),"")</f>
@@ -5490,7 +5490,7 @@
         <v>356.53</v>
       </c>
       <c r="L38" s="5" t="n">
-        <v>378.465</v>
+        <v>378.510009765625</v>
       </c>
       <c r="M38" s="7">
         <f>IFERROR(IF(E38="Short",-1,1)*(IF(K38&lt;&gt;"",K38,L38)/J38-1),"")</f>
@@ -5565,7 +5565,7 @@
         <v>344.42</v>
       </c>
       <c r="L39" s="5" t="n">
-        <v>337.87</v>
+        <v>337.7999877929688</v>
       </c>
       <c r="M39" s="7">
         <f>IFERROR(IF(E39="Short",-1,1)*(IF(K39&lt;&gt;"",K39,L39)/J39-1),"")</f>
@@ -5636,7 +5636,7 @@
         <v>188.498788</v>
       </c>
       <c r="L40" s="5" t="n">
-        <v>192.27</v>
+        <v>192.2799987792969</v>
       </c>
       <c r="M40" s="7">
         <f>IFERROR(IF(E40="Short",-1,1)*(IF(K40&lt;&gt;"",K40,L40)/J40-1),"")</f>
@@ -5707,7 +5707,7 @@
         <v>526.15</v>
       </c>
       <c r="L41" s="5" t="n">
-        <v>540.62</v>
+        <v>538.989990234375</v>
       </c>
       <c r="M41" s="7">
         <f>IFERROR(IF(E41="Short",-1,1)*(IF(K41&lt;&gt;"",K41,L41)/J41-1),"")</f>
@@ -5778,7 +5778,7 @@
         <v>276.52</v>
       </c>
       <c r="L42" s="5" t="n">
-        <v>270.63</v>
+        <v>270.739990234375</v>
       </c>
       <c r="M42" s="7">
         <f>IFERROR(IF(E42="Short",-1,1)*(IF(K42&lt;&gt;"",K42,L42)/J42-1),"")</f>
@@ -5843,7 +5843,7 @@
         <v>349.461111</v>
       </c>
       <c r="L43" s="5" t="n">
-        <v>334.715</v>
+        <v>334.760009765625</v>
       </c>
       <c r="M43" s="7">
         <f>IFERROR(IF(E43="Short",-1,1)*(IF(K43&lt;&gt;"",K43,L43)/J43-1),"")</f>
@@ -5914,7 +5914,7 @@
         <v>869.4233330000001</v>
       </c>
       <c r="L44" s="5" t="n">
-        <v>851.22</v>
+        <v>850.7000122070312</v>
       </c>
       <c r="M44" s="7">
         <f>IFERROR(IF(E44="Short",-1,1)*(IF(K44&lt;&gt;"",K44,L44)/J44-1),"")</f>
@@ -5985,7 +5985,7 @@
         <v>1253.68</v>
       </c>
       <c r="L45" s="5" t="n">
-        <v>1270.89</v>
+        <v>1270.75</v>
       </c>
       <c r="M45" s="7">
         <f>IFERROR(IF(E45="Short",-1,1)*(IF(K45&lt;&gt;"",K45,L45)/J45-1),"")</f>
@@ -6056,7 +6056,7 @@
         <v>99.13124999999999</v>
       </c>
       <c r="L46" s="5" t="n">
-        <v>96.535</v>
+        <v>96.52999877929688</v>
       </c>
       <c r="M46" s="7">
         <f>IFERROR(IF(E46="Short",-1,1)*(IF(K46&lt;&gt;"",K46,L46)/J46-1),"")</f>
@@ -6121,7 +6121,7 @@
         <v>242.642308</v>
       </c>
       <c r="L47" s="5" t="n">
-        <v>246.245</v>
+        <v>246.25</v>
       </c>
       <c r="M47" s="7">
         <f>IFERROR(IF(E47="Short",-1,1)*(IF(K47&lt;&gt;"",K47,L47)/J47-1),"")</f>
@@ -6186,7 +6186,7 @@
         <v>736.4924999999999</v>
       </c>
       <c r="L48" s="5" t="n">
-        <v>718.9400000000001</v>
+        <v>697.52001953125</v>
       </c>
       <c r="M48" s="7">
         <f>IFERROR(IF(E48="Short",-1,1)*(IF(K48&lt;&gt;"",K48,L48)/J48-1),"")</f>
@@ -6257,7 +6257,7 @@
         <v>128.4175</v>
       </c>
       <c r="L49" s="5" t="n">
-        <v>134.69</v>
+        <v>134.6999969482422</v>
       </c>
       <c r="M49" s="7">
         <f>IFERROR(IF(E49="Short",-1,1)*(IF(K49&lt;&gt;"",K49,L49)/J49-1),"")</f>
@@ -6322,7 +6322,7 @@
         <v>1395.31</v>
       </c>
       <c r="L50" s="5" t="n">
-        <v>1379.57</v>
+        <v>1378.219970703125</v>
       </c>
       <c r="M50" s="7">
         <f>IFERROR(IF(E50="Short",-1,1)*(IF(K50&lt;&gt;"",K50,L50)/J50-1),"")</f>
@@ -6393,7 +6393,7 @@
         <v>771.98</v>
       </c>
       <c r="L51" s="5" t="n">
-        <v>773.22</v>
+        <v>773.0900268554688</v>
       </c>
       <c r="M51" s="7">
         <f>IFERROR(IF(E51="Short",-1,1)*(IF(K51&lt;&gt;"",K51,L51)/J51-1),"")</f>
@@ -6462,7 +6462,7 @@
         <v>691.4699999999999</v>
       </c>
       <c r="L52" s="5" t="n">
-        <v>697.38</v>
+        <v>696.8900146484375</v>
       </c>
       <c r="M52" s="7">
         <f>IFERROR(IF(E52="Short",-1,1)*(IF(K52&lt;&gt;"",K52,L52)/J52-1),"")</f>
@@ -6533,7 +6533,7 @@
         <v>356.53</v>
       </c>
       <c r="L53" s="5" t="n">
-        <v>378.465</v>
+        <v>378.510009765625</v>
       </c>
       <c r="M53" s="7">
         <f>IFERROR(IF(E53="Short",-1,1)*(IF(K53&lt;&gt;"",K53,L53)/J53-1),"")</f>
@@ -6598,7 +6598,7 @@
         <v>32.45</v>
       </c>
       <c r="L54" s="5" t="n">
-        <v>35.55</v>
+        <v>35.56999969482422</v>
       </c>
       <c r="M54" s="7">
         <f>IFERROR(IF(E54="Short",-1,1)*(IF(K54&lt;&gt;"",K54,L54)/J54-1),"")</f>
@@ -6669,7 +6669,7 @@
         <v>317.94</v>
       </c>
       <c r="L55" s="5" t="n">
-        <v>320.495</v>
+        <v>320.5499877929688</v>
       </c>
       <c r="M55" s="7">
         <f>IFERROR(IF(E55="Short",-1,1)*(IF(K55&lt;&gt;"",K55,L55)/J55-1),"")</f>
@@ -6740,7 +6740,7 @@
         <v>533.04</v>
       </c>
       <c r="L56" s="5" t="n">
-        <v>532.8</v>
+        <v>532.9500122070312</v>
       </c>
       <c r="M56" s="7">
         <f>IFERROR(IF(E56="Short",-1,1)*(IF(K56&lt;&gt;"",K56,L56)/J56-1),"")</f>
@@ -6811,7 +6811,7 @@
         <v>65.068667</v>
       </c>
       <c r="L57" s="5" t="n">
-        <v>65.05</v>
+        <v>65.04000091552734</v>
       </c>
       <c r="M57" s="7">
         <f>IFERROR(IF(E57="Short",-1,1)*(IF(K57&lt;&gt;"",K57,L57)/J57-1),"")</f>
@@ -6882,7 +6882,7 @@
         <v>221.922727</v>
       </c>
       <c r="L58" s="5" t="n">
-        <v>221.9</v>
+        <v>221.9700012207031</v>
       </c>
       <c r="M58" s="7">
         <f>IFERROR(IF(E58="Short",-1,1)*(IF(K58&lt;&gt;"",K58,L58)/J58-1),"")</f>
@@ -6953,7 +6953,7 @@
         <v>76.93108100000001</v>
       </c>
       <c r="L59" s="5" t="n">
-        <v>76.93000000000001</v>
+        <v>76.94000244140625</v>
       </c>
       <c r="M59" s="7">
         <f>IFERROR(IF(E59="Short",-1,1)*(IF(K59&lt;&gt;"",K59,L59)/J59-1),"")</f>
@@ -7024,7 +7024,7 @@
         <v>129.046897</v>
       </c>
       <c r="L60" s="5" t="n">
-        <v>129.09</v>
+        <v>129.1300048828125</v>
       </c>
       <c r="M60" s="7">
         <f>IFERROR(IF(E60="Short",-1,1)*(IF(K60&lt;&gt;"",K60,L60)/J60-1),"")</f>
@@ -7095,7 +7095,7 @@
         <v>386.4025</v>
       </c>
       <c r="L61" s="5" t="n">
-        <v>392.72</v>
+        <v>386.4700012207031</v>
       </c>
       <c r="M61" s="7">
         <f>IFERROR(IF(E61="Short",-1,1)*(IF(K61&lt;&gt;"",K61,L61)/J61-1),"")</f>
@@ -7160,7 +7160,7 @@
       </c>
       <c r="K62" s="5" t="n"/>
       <c r="L62" s="5" t="n">
-        <v>553.78</v>
+        <v>552.719970703125</v>
       </c>
       <c r="M62" s="7">
         <f>IFERROR(IF(E62="Short",-1,1)*(IF(K62&lt;&gt;"",K62,L62)/J62-1),"")</f>
@@ -7225,7 +7225,7 @@
       </c>
       <c r="K63" s="5" t="n"/>
       <c r="L63" s="5" t="n">
-        <v>58.17</v>
+        <v>58.16999816894531</v>
       </c>
       <c r="M63" s="7">
         <f>IFERROR(IF(E63="Short",-1,1)*(IF(K63&lt;&gt;"",K63,L63)/J63-1),"")</f>
@@ -7290,7 +7290,7 @@
       </c>
       <c r="K64" s="5" t="n"/>
       <c r="L64" s="5" t="n">
-        <v>244.66</v>
+        <v>244.7599945068359</v>
       </c>
       <c r="M64" s="7">
         <f>IFERROR(IF(E64="Short",-1,1)*(IF(K64&lt;&gt;"",K64,L64)/J64-1),"")</f>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="K65" s="5" t="n"/>
       <c r="L65" s="5" t="n">
-        <v>37.525</v>
+        <v>37.52999877929688</v>
       </c>
       <c r="M65" s="7">
         <f>IFERROR(IF(E65="Short",-1,1)*(IF(K65&lt;&gt;"",K65,L65)/J65-1),"")</f>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="K66" s="5" t="n"/>
       <c r="L66" s="5" t="n">
-        <v>773.22</v>
+        <v>773.0900268554688</v>
       </c>
       <c r="M66" s="7">
         <f>IFERROR(IF(E66="Short",-1,1)*(IF(K66&lt;&gt;"",K66,L66)/J66-1),"")</f>
@@ -7483,7 +7483,7 @@
       </c>
       <c r="K67" s="5" t="n"/>
       <c r="L67" s="5" t="n">
-        <v>50.81</v>
+        <v>50.77999877929688</v>
       </c>
       <c r="M67" s="7">
         <f>IFERROR(IF(E67="Short",-1,1)*(IF(K67&lt;&gt;"",K67,L67)/J67-1),"")</f>
@@ -7548,7 +7548,7 @@
       </c>
       <c r="K68" s="5" t="n"/>
       <c r="L68" s="5" t="n">
-        <v>241.75</v>
+        <v>241.7799987792969</v>
       </c>
       <c r="M68" s="7">
         <f>IFERROR(IF(E68="Short",-1,1)*(IF(K68&lt;&gt;"",K68,L68)/J68-1),"")</f>
@@ -7613,7 +7613,7 @@
       </c>
       <c r="K69" s="5" t="n"/>
       <c r="L69" s="5" t="n">
-        <v>77.68000000000001</v>
+        <v>77.66999816894531</v>
       </c>
       <c r="M69" s="7">
         <f>IFERROR(IF(E69="Short",-1,1)*(IF(K69&lt;&gt;"",K69,L69)/J69-1),"")</f>
@@ -7678,7 +7678,7 @@
       </c>
       <c r="K70" s="5" t="n"/>
       <c r="L70" s="5" t="n">
-        <v>335.11</v>
+        <v>335.1900024414062</v>
       </c>
       <c r="M70" s="7">
         <f>IFERROR(IF(E70="Short",-1,1)*(IF(K70&lt;&gt;"",K70,L70)/J70-1),"")</f>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="K71" s="5" t="n"/>
       <c r="L71" s="5" t="n">
-        <v>23.505</v>
+        <v>23.5</v>
       </c>
       <c r="M71" s="7">
         <f>IFERROR(IF(E71="Short",-1,1)*(IF(K71&lt;&gt;"",K71,L71)/J71-1),"")</f>
@@ -7808,7 +7808,7 @@
       </c>
       <c r="K72" s="5" t="n"/>
       <c r="L72" s="5" t="n">
-        <v>168.7</v>
+        <v>168.9499969482422</v>
       </c>
       <c r="M72" s="7">
         <f>IFERROR(IF(E72="Short",-1,1)*(IF(K72&lt;&gt;"",K72,L72)/J72-1),"")</f>

</xml_diff>

<commit_message>
fund memo + performance 2026-10-29T00:06Z
</commit_message>
<xml_diff>
--- a/fund_state/live/ledger/fund_positions.xlsx
+++ b/fund_state/live/ledger/fund_positions.xlsx
@@ -490,11 +490,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Account value (Alpaca, 2026-10-28 16:16 ET)</t>
+          <t>Account value (Alpaca, 2026-10-28 20:06 ET)</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>98930.67819999999</v>
+        <v>98798.44</v>
       </c>
     </row>
     <row r="3">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1406.468199999999</v>
+        <v>1274.229999999999</v>
       </c>
     </row>
     <row r="7">
@@ -666,7 +666,7 @@
         <v>348.1885714285714</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>344.3</v>
+        <v>345.5</v>
       </c>
       <c r="H2" s="6">
         <f>D2*G2</f>
@@ -709,7 +709,7 @@
         <v>28.07</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>29.4663</v>
+        <v>30.74</v>
       </c>
       <c r="H3" s="6">
         <f>D3*G3</f>
@@ -752,7 +752,7 @@
         <v>51.40897142857144</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>52.7</v>
+        <v>52.89</v>
       </c>
       <c r="H4" s="6">
         <f>D4*G4</f>
@@ -838,7 +838,7 @@
         <v>230.03</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>255.59</v>
+        <v>249.67</v>
       </c>
       <c r="H6" s="6">
         <f>D6*G6</f>
@@ -881,7 +881,7 @@
         <v>520.91</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>553.71</v>
+        <v>545.99</v>
       </c>
       <c r="H7" s="6">
         <f>D7*G7</f>
@@ -924,7 +924,7 @@
         <v>65.86089552238806</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>62.13</v>
+        <v>62.3</v>
       </c>
       <c r="H8" s="6">
         <f>D8*G8</f>
@@ -967,7 +967,7 @@
         <v>35.04272084805654</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>33.45</v>
+        <v>33.5</v>
       </c>
       <c r="H9" s="6">
         <f>D9*G9</f>
@@ -1010,7 +1010,7 @@
         <v>33.4584962406015</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>35.45</v>
+        <v>34.95</v>
       </c>
       <c r="H10" s="6">
         <f>D10*G10</f>
@@ -1053,7 +1053,7 @@
         <v>765.3002702702703</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>771.74</v>
+        <v>769.59</v>
       </c>
       <c r="H11" s="6">
         <f>D11*G11</f>
@@ -1096,7 +1096,7 @@
         <v>374.146</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>403.82</v>
+        <v>401.39</v>
       </c>
       <c r="H12" s="6">
         <f>D12*G12</f>
@@ -3590,7 +3590,7 @@
         <v>773.95</v>
       </c>
       <c r="L2" s="5" t="n">
-        <v>773.08</v>
+        <v>769.6599731445312</v>
       </c>
       <c r="M2" s="7">
         <f>IFERROR(IF(E2="Short",-1,1)*(IF(K2&lt;&gt;"",K2,L2)/J2-1),"")</f>
@@ -3659,7 +3659,7 @@
         <v>998.54</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>878.705</v>
+        <v>895.0800170898438</v>
       </c>
       <c r="M3" s="7">
         <f>IFERROR(IF(E3="Short",-1,1)*(IF(K3&lt;&gt;"",K3,L3)/J3-1),"")</f>
@@ -3734,7 +3734,7 @@
         <v>1086.75</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>978.25</v>
+        <v>928.760009765625</v>
       </c>
       <c r="M4" s="7">
         <f>IFERROR(IF(E4="Short",-1,1)*(IF(K4&lt;&gt;"",K4,L4)/J4-1),"")</f>
@@ -3809,7 +3809,7 @@
         <v>1036.16</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>978.25</v>
+        <v>928.760009765625</v>
       </c>
       <c r="M5" s="7">
         <f>IFERROR(IF(E5="Short",-1,1)*(IF(K5&lt;&gt;"",K5,L5)/J5-1),"")</f>
@@ -3884,7 +3884,7 @@
         <v>71.59</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>62</v>
+        <v>62.52000045776367</v>
       </c>
       <c r="M6" s="7">
         <f>IFERROR(IF(E6="Short",-1,1)*(IF(K6&lt;&gt;"",K6,L6)/J6-1),"")</f>
@@ -3959,7 +3959,7 @@
         <v>511.0499877929688</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>540.8099999999999</v>
+        <v>542.989990234375</v>
       </c>
       <c r="M7" s="7">
         <f>IFERROR(IF(E7="Short",-1,1)*(IF(K7&lt;&gt;"",K7,L7)/J7-1),"")</f>
@@ -4034,7 +4034,7 @@
         <v>92.70999999999999</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>105.24</v>
+        <v>104.5899963378906</v>
       </c>
       <c r="M8" s="7">
         <f>IFERROR(IF(E8="Short",-1,1)*(IF(K8&lt;&gt;"",K8,L8)/J8-1),"")</f>
@@ -4109,7 +4109,7 @@
         <v>118.22</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>129.805</v>
+        <v>130.6300048828125</v>
       </c>
       <c r="M9" s="7">
         <f>IFERROR(IF(E9="Short",-1,1)*(IF(K9&lt;&gt;"",K9,L9)/J9-1),"")</f>
@@ -4184,7 +4184,7 @@
         <v>778.28</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>773.08</v>
+        <v>769.6599731445312</v>
       </c>
       <c r="M10" s="7">
         <f>IFERROR(IF(E10="Short",-1,1)*(IF(K10&lt;&gt;"",K10,L10)/J10-1),"")</f>
@@ -4253,7 +4253,7 @@
         <v>777.915</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>773.08</v>
+        <v>769.6599731445312</v>
       </c>
       <c r="M11" s="7">
         <f>IFERROR(IF(E11="Short",-1,1)*(IF(K11&lt;&gt;"",K11,L11)/J11-1),"")</f>
@@ -4322,7 +4322,7 @@
         <v>768.885</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>773.08</v>
+        <v>769.6599731445312</v>
       </c>
       <c r="M12" s="7">
         <f>IFERROR(IF(E12="Short",-1,1)*(IF(K12&lt;&gt;"",K12,L12)/J12-1),"")</f>
@@ -4391,7 +4391,7 @@
         <v>771.98</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>773.08</v>
+        <v>769.6599731445312</v>
       </c>
       <c r="M13" s="7">
         <f>IFERROR(IF(E13="Short",-1,1)*(IF(K13&lt;&gt;"",K13,L13)/J13-1),"")</f>
@@ -4460,7 +4460,7 @@
         <v>605.795</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>578.4349999999999</v>
+        <v>560.260009765625</v>
       </c>
       <c r="M14" s="7">
         <f>IFERROR(IF(E14="Short",-1,1)*(IF(K14&lt;&gt;"",K14,L14)/J14-1),"")</f>
@@ -4535,7 +4535,7 @@
         <v>562.54</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>578.4349999999999</v>
+        <v>560.260009765625</v>
       </c>
       <c r="M15" s="7">
         <f>IFERROR(IF(E15="Short",-1,1)*(IF(K15&lt;&gt;"",K15,L15)/J15-1),"")</f>
@@ -4610,7 +4610,7 @@
         <v>361.53</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>351.9</v>
+        <v>342.3299865722656</v>
       </c>
       <c r="M16" s="7">
         <f>IFERROR(IF(E16="Short",-1,1)*(IF(K16&lt;&gt;"",K16,L16)/J16-1),"")</f>
@@ -4685,7 +4685,7 @@
         <v>357.595</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>351.9</v>
+        <v>342.3299865722656</v>
       </c>
       <c r="M17" s="7">
         <f>IFERROR(IF(E17="Short",-1,1)*(IF(K17&lt;&gt;"",K17,L17)/J17-1),"")</f>
@@ -4760,7 +4760,7 @@
         <v>344.42</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>351.9</v>
+        <v>342.3299865722656</v>
       </c>
       <c r="M18" s="7">
         <f>IFERROR(IF(E18="Short",-1,1)*(IF(K18&lt;&gt;"",K18,L18)/J18-1),"")</f>
@@ -4835,7 +4835,7 @@
         <v>188.498788</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>166.98</v>
+        <v>168.1799926757812</v>
       </c>
       <c r="M19" s="7">
         <f>IFERROR(IF(E19="Short",-1,1)*(IF(K19&lt;&gt;"",K19,L19)/J19-1),"")</f>
@@ -4910,7 +4910,7 @@
         <v>276.52</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>258.175</v>
+        <v>258.9800109863281</v>
       </c>
       <c r="M20" s="7">
         <f>IFERROR(IF(E20="Short",-1,1)*(IF(K20&lt;&gt;"",K20,L20)/J20-1),"")</f>
@@ -4985,7 +4985,7 @@
         <v>349.461111</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>301.74</v>
+        <v>320.5799865722656</v>
       </c>
       <c r="M21" s="7">
         <f>IFERROR(IF(E21="Short",-1,1)*(IF(K21&lt;&gt;"",K21,L21)/J21-1),"")</f>
@@ -5060,7 +5060,7 @@
         <v>58.7</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>60.34</v>
+        <v>60.84000015258789</v>
       </c>
       <c r="M22" s="7">
         <f>IFERROR(IF(E22="Short",-1,1)*(IF(K22&lt;&gt;"",K22,L22)/J22-1),"")</f>
@@ -5135,7 +5135,7 @@
         <v>869.4233330000001</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>913.8049999999999</v>
+        <v>866.1799926757812</v>
       </c>
       <c r="M23" s="7">
         <f>IFERROR(IF(E23="Short",-1,1)*(IF(K23&lt;&gt;"",K23,L23)/J23-1),"")</f>
@@ -5210,7 +5210,7 @@
         <v>1253.68</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>1290.67</v>
+        <v>1281.910034179688</v>
       </c>
       <c r="M24" s="7">
         <f>IFERROR(IF(E24="Short",-1,1)*(IF(K24&lt;&gt;"",K24,L24)/J24-1),"")</f>
@@ -5285,7 +5285,7 @@
         <v>241.535</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>251.73</v>
+        <v>243.5700073242188</v>
       </c>
       <c r="M25" s="7">
         <f>IFERROR(IF(E25="Short",-1,1)*(IF(K25&lt;&gt;"",K25,L25)/J25-1),"")</f>
@@ -5360,7 +5360,7 @@
         <v>221.17</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>215.07</v>
+        <v>217.9400024414062</v>
       </c>
       <c r="M26" s="7">
         <f>IFERROR(IF(E26="Short",-1,1)*(IF(K26&lt;&gt;"",K26,L26)/J26-1),"")</f>
@@ -5435,7 +5435,7 @@
         <v>217.33</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>215.07</v>
+        <v>217.9400024414062</v>
       </c>
       <c r="M27" s="7">
         <f>IFERROR(IF(E27="Short",-1,1)*(IF(K27&lt;&gt;"",K27,L27)/J27-1),"")</f>
@@ -5510,7 +5510,7 @@
         <v>526.15</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>540.8099999999999</v>
+        <v>542.989990234375</v>
       </c>
       <c r="M28" s="7">
         <f>IFERROR(IF(E28="Short",-1,1)*(IF(K28&lt;&gt;"",K28,L28)/J28-1),"")</f>
@@ -5585,7 +5585,7 @@
         <v>99.13124999999999</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>105.24</v>
+        <v>104.5899963378906</v>
       </c>
       <c r="M29" s="7">
         <f>IFERROR(IF(E29="Short",-1,1)*(IF(K29&lt;&gt;"",K29,L29)/J29-1),"")</f>
@@ -5660,7 +5660,7 @@
         <v>242.642308</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>250.625</v>
+        <v>249.4700012207031</v>
       </c>
       <c r="M30" s="7">
         <f>IFERROR(IF(E30="Short",-1,1)*(IF(K30&lt;&gt;"",K30,L30)/J30-1),"")</f>
@@ -5735,7 +5735,7 @@
         <v>736.4924999999999</v>
       </c>
       <c r="L31" s="5" t="n">
-        <v>614.08</v>
+        <v>620.1900024414062</v>
       </c>
       <c r="M31" s="7">
         <f>IFERROR(IF(E31="Short",-1,1)*(IF(K31&lt;&gt;"",K31,L31)/J31-1),"")</f>
@@ -5810,7 +5810,7 @@
         <v>37.13999938964844</v>
       </c>
       <c r="L32" s="5" t="n">
-        <v>37.165</v>
+        <v>37.56000137329102</v>
       </c>
       <c r="M32" s="7">
         <f>IFERROR(IF(E32="Short",-1,1)*(IF(K32&lt;&gt;"",K32,L32)/J32-1),"")</f>
@@ -5885,7 +5885,7 @@
         <v>125.99375</v>
       </c>
       <c r="L33" s="5" t="n">
-        <v>132.66</v>
+        <v>133.5</v>
       </c>
       <c r="M33" s="7">
         <f>IFERROR(IF(E33="Short",-1,1)*(IF(K33&lt;&gt;"",K33,L33)/J33-1),"")</f>
@@ -5960,7 +5960,7 @@
         <v>128.4175</v>
       </c>
       <c r="L34" s="5" t="n">
-        <v>132.66</v>
+        <v>133.5</v>
       </c>
       <c r="M34" s="7">
         <f>IFERROR(IF(E34="Short",-1,1)*(IF(K34&lt;&gt;"",K34,L34)/J34-1),"")</f>
@@ -6035,7 +6035,7 @@
         <v>1581.73</v>
       </c>
       <c r="L35" s="5" t="n">
-        <v>1392.72</v>
+        <v>1304.839965820312</v>
       </c>
       <c r="M35" s="7">
         <f>IFERROR(IF(E35="Short",-1,1)*(IF(K35&lt;&gt;"",K35,L35)/J35-1),"")</f>
@@ -6110,7 +6110,7 @@
         <v>1395.31</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>1392.72</v>
+        <v>1304.839965820312</v>
       </c>
       <c r="M36" s="7">
         <f>IFERROR(IF(E36="Short",-1,1)*(IF(K36&lt;&gt;"",K36,L36)/J36-1),"")</f>
@@ -6185,7 +6185,7 @@
         <v>691.4699999999999</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>698.0599999999999</v>
+        <v>667.8499755859375</v>
       </c>
       <c r="M37" s="7">
         <f>IFERROR(IF(E37="Short",-1,1)*(IF(K37&lt;&gt;"",K37,L37)/J37-1),"")</f>
@@ -6260,7 +6260,7 @@
         <v>356.53</v>
       </c>
       <c r="L38" s="5" t="n">
-        <v>396.45</v>
+        <v>380.8800048828125</v>
       </c>
       <c r="M38" s="7">
         <f>IFERROR(IF(E38="Short",-1,1)*(IF(K38&lt;&gt;"",K38,L38)/J38-1),"")</f>
@@ -6335,7 +6335,7 @@
         <v>344.42</v>
       </c>
       <c r="L39" s="5" t="n">
-        <v>351.9</v>
+        <v>342.3299865722656</v>
       </c>
       <c r="M39" s="7">
         <f>IFERROR(IF(E39="Short",-1,1)*(IF(K39&lt;&gt;"",K39,L39)/J39-1),"")</f>
@@ -6406,7 +6406,7 @@
         <v>188.498788</v>
       </c>
       <c r="L40" s="5" t="n">
-        <v>166.98</v>
+        <v>168.1799926757812</v>
       </c>
       <c r="M40" s="7">
         <f>IFERROR(IF(E40="Short",-1,1)*(IF(K40&lt;&gt;"",K40,L40)/J40-1),"")</f>
@@ -6477,7 +6477,7 @@
         <v>526.15</v>
       </c>
       <c r="L41" s="5" t="n">
-        <v>540.8099999999999</v>
+        <v>542.989990234375</v>
       </c>
       <c r="M41" s="7">
         <f>IFERROR(IF(E41="Short",-1,1)*(IF(K41&lt;&gt;"",K41,L41)/J41-1),"")</f>
@@ -6548,7 +6548,7 @@
         <v>276.52</v>
       </c>
       <c r="L42" s="5" t="n">
-        <v>258.175</v>
+        <v>258.9800109863281</v>
       </c>
       <c r="M42" s="7">
         <f>IFERROR(IF(E42="Short",-1,1)*(IF(K42&lt;&gt;"",K42,L42)/J42-1),"")</f>
@@ -6613,7 +6613,7 @@
         <v>349.461111</v>
       </c>
       <c r="L43" s="5" t="n">
-        <v>301.74</v>
+        <v>320.5799865722656</v>
       </c>
       <c r="M43" s="7">
         <f>IFERROR(IF(E43="Short",-1,1)*(IF(K43&lt;&gt;"",K43,L43)/J43-1),"")</f>
@@ -6684,7 +6684,7 @@
         <v>869.4233330000001</v>
       </c>
       <c r="L44" s="5" t="n">
-        <v>913.8049999999999</v>
+        <v>866.1799926757812</v>
       </c>
       <c r="M44" s="7">
         <f>IFERROR(IF(E44="Short",-1,1)*(IF(K44&lt;&gt;"",K44,L44)/J44-1),"")</f>
@@ -6755,7 +6755,7 @@
         <v>1253.68</v>
       </c>
       <c r="L45" s="5" t="n">
-        <v>1290.67</v>
+        <v>1281.910034179688</v>
       </c>
       <c r="M45" s="7">
         <f>IFERROR(IF(E45="Short",-1,1)*(IF(K45&lt;&gt;"",K45,L45)/J45-1),"")</f>
@@ -6826,7 +6826,7 @@
         <v>99.13124999999999</v>
       </c>
       <c r="L46" s="5" t="n">
-        <v>105.24</v>
+        <v>104.5899963378906</v>
       </c>
       <c r="M46" s="7">
         <f>IFERROR(IF(E46="Short",-1,1)*(IF(K46&lt;&gt;"",K46,L46)/J46-1),"")</f>
@@ -6891,7 +6891,7 @@
         <v>242.642308</v>
       </c>
       <c r="L47" s="5" t="n">
-        <v>250.625</v>
+        <v>249.4700012207031</v>
       </c>
       <c r="M47" s="7">
         <f>IFERROR(IF(E47="Short",-1,1)*(IF(K47&lt;&gt;"",K47,L47)/J47-1),"")</f>
@@ -6956,7 +6956,7 @@
         <v>736.4924999999999</v>
       </c>
       <c r="L48" s="5" t="n">
-        <v>614.08</v>
+        <v>620.1900024414062</v>
       </c>
       <c r="M48" s="7">
         <f>IFERROR(IF(E48="Short",-1,1)*(IF(K48&lt;&gt;"",K48,L48)/J48-1),"")</f>
@@ -7027,7 +7027,7 @@
         <v>128.4175</v>
       </c>
       <c r="L49" s="5" t="n">
-        <v>132.66</v>
+        <v>133.5</v>
       </c>
       <c r="M49" s="7">
         <f>IFERROR(IF(E49="Short",-1,1)*(IF(K49&lt;&gt;"",K49,L49)/J49-1),"")</f>
@@ -7092,7 +7092,7 @@
         <v>1395.31</v>
       </c>
       <c r="L50" s="5" t="n">
-        <v>1392.72</v>
+        <v>1304.839965820312</v>
       </c>
       <c r="M50" s="7">
         <f>IFERROR(IF(E50="Short",-1,1)*(IF(K50&lt;&gt;"",K50,L50)/J50-1),"")</f>
@@ -7163,7 +7163,7 @@
         <v>771.98</v>
       </c>
       <c r="L51" s="5" t="n">
-        <v>773.08</v>
+        <v>769.6599731445312</v>
       </c>
       <c r="M51" s="7">
         <f>IFERROR(IF(E51="Short",-1,1)*(IF(K51&lt;&gt;"",K51,L51)/J51-1),"")</f>
@@ -7232,7 +7232,7 @@
         <v>691.4699999999999</v>
       </c>
       <c r="L52" s="5" t="n">
-        <v>698.0599999999999</v>
+        <v>667.8499755859375</v>
       </c>
       <c r="M52" s="7">
         <f>IFERROR(IF(E52="Short",-1,1)*(IF(K52&lt;&gt;"",K52,L52)/J52-1),"")</f>
@@ -7303,7 +7303,7 @@
         <v>356.53</v>
       </c>
       <c r="L53" s="5" t="n">
-        <v>396.45</v>
+        <v>380.8800048828125</v>
       </c>
       <c r="M53" s="7">
         <f>IFERROR(IF(E53="Short",-1,1)*(IF(K53&lt;&gt;"",K53,L53)/J53-1),"")</f>
@@ -7368,7 +7368,7 @@
         <v>32.45</v>
       </c>
       <c r="L54" s="5" t="n">
-        <v>35.83</v>
+        <v>35.09000015258789</v>
       </c>
       <c r="M54" s="7">
         <f>IFERROR(IF(E54="Short",-1,1)*(IF(K54&lt;&gt;"",K54,L54)/J54-1),"")</f>
@@ -7439,7 +7439,7 @@
         <v>317.94</v>
       </c>
       <c r="L55" s="5" t="n">
-        <v>317.91</v>
+        <v>313.4599914550781</v>
       </c>
       <c r="M55" s="7">
         <f>IFERROR(IF(E55="Short",-1,1)*(IF(K55&lt;&gt;"",K55,L55)/J55-1),"")</f>
@@ -7510,7 +7510,7 @@
         <v>533.04</v>
       </c>
       <c r="L56" s="5" t="n">
-        <v>551.54</v>
+        <v>531.3300170898438</v>
       </c>
       <c r="M56" s="7">
         <f>IFERROR(IF(E56="Short",-1,1)*(IF(K56&lt;&gt;"",K56,L56)/J56-1),"")</f>
@@ -7581,7 +7581,7 @@
         <v>65.068667</v>
       </c>
       <c r="L57" s="5" t="n">
-        <v>62</v>
+        <v>62.52000045776367</v>
       </c>
       <c r="M57" s="7">
         <f>IFERROR(IF(E57="Short",-1,1)*(IF(K57&lt;&gt;"",K57,L57)/J57-1),"")</f>
@@ -7652,7 +7652,7 @@
         <v>221.922727</v>
       </c>
       <c r="L58" s="5" t="n">
-        <v>215.07</v>
+        <v>217.9400024414062</v>
       </c>
       <c r="M58" s="7">
         <f>IFERROR(IF(E58="Short",-1,1)*(IF(K58&lt;&gt;"",K58,L58)/J58-1),"")</f>
@@ -7723,7 +7723,7 @@
         <v>76.93108100000001</v>
       </c>
       <c r="L59" s="5" t="n">
-        <v>75.63</v>
+        <v>78.66999816894531</v>
       </c>
       <c r="M59" s="7">
         <f>IFERROR(IF(E59="Short",-1,1)*(IF(K59&lt;&gt;"",K59,L59)/J59-1),"")</f>
@@ -7794,7 +7794,7 @@
         <v>129.046897</v>
       </c>
       <c r="L60" s="5" t="n">
-        <v>144.29</v>
+        <v>130.5299987792969</v>
       </c>
       <c r="M60" s="7">
         <f>IFERROR(IF(E60="Short",-1,1)*(IF(K60&lt;&gt;"",K60,L60)/J60-1),"")</f>
@@ -7865,7 +7865,7 @@
         <v>386.4025</v>
       </c>
       <c r="L61" s="5" t="n">
-        <v>403.5</v>
+        <v>407.4599914550781</v>
       </c>
       <c r="M61" s="7">
         <f>IFERROR(IF(E61="Short",-1,1)*(IF(K61&lt;&gt;"",K61,L61)/J61-1),"")</f>
@@ -7936,7 +7936,7 @@
         <v>508.143333</v>
       </c>
       <c r="L62" s="5" t="n">
-        <v>578.4349999999999</v>
+        <v>560.260009765625</v>
       </c>
       <c r="M62" s="7">
         <f>IFERROR(IF(E62="Short",-1,1)*(IF(K62&lt;&gt;"",K62,L62)/J62-1),"")</f>
@@ -8007,7 +8007,7 @@
         <v>51.03</v>
       </c>
       <c r="L63" s="5" t="n">
-        <v>50.88</v>
+        <v>50.68000030517578</v>
       </c>
       <c r="M63" s="7">
         <f>IFERROR(IF(E63="Short",-1,1)*(IF(K63&lt;&gt;"",K63,L63)/J63-1),"")</f>
@@ -8078,7 +8078,7 @@
         <v>250.53</v>
       </c>
       <c r="L64" s="5" t="n">
-        <v>242.4</v>
+        <v>240.8899993896484</v>
       </c>
       <c r="M64" s="7">
         <f>IFERROR(IF(E64="Short",-1,1)*(IF(K64&lt;&gt;"",K64,L64)/J64-1),"")</f>
@@ -8149,7 +8149,7 @@
         <v>79.149362</v>
       </c>
       <c r="L65" s="5" t="n">
-        <v>80.36</v>
+        <v>81.44999694824219</v>
       </c>
       <c r="M65" s="7">
         <f>IFERROR(IF(E65="Short",-1,1)*(IF(K65&lt;&gt;"",K65,L65)/J65-1),"")</f>
@@ -8220,7 +8220,7 @@
         <v>55.43</v>
       </c>
       <c r="L66" s="5" t="n">
-        <v>60.34</v>
+        <v>60.84000015258789</v>
       </c>
       <c r="M66" s="7">
         <f>IFERROR(IF(E66="Short",-1,1)*(IF(K66&lt;&gt;"",K66,L66)/J66-1),"")</f>
@@ -8291,7 +8291,7 @@
         <v>336.362857</v>
       </c>
       <c r="L67" s="5" t="n">
-        <v>339.405</v>
+        <v>335.7900085449219</v>
       </c>
       <c r="M67" s="7">
         <f>IFERROR(IF(E67="Short",-1,1)*(IF(K67&lt;&gt;"",K67,L67)/J67-1),"")</f>
@@ -8362,7 +8362,7 @@
         <v>25.1</v>
       </c>
       <c r="L68" s="5" t="n">
-        <v>23.88</v>
+        <v>24.05999946594238</v>
       </c>
       <c r="M68" s="7">
         <f>IFERROR(IF(E68="Short",-1,1)*(IF(K68&lt;&gt;"",K68,L68)/J68-1),"")</f>
@@ -8433,7 +8433,7 @@
         <v>167.732857</v>
       </c>
       <c r="L69" s="5" t="n">
-        <v>173.605</v>
+        <v>170.8899993896484</v>
       </c>
       <c r="M69" s="7">
         <f>IFERROR(IF(E69="Short",-1,1)*(IF(K69&lt;&gt;"",K69,L69)/J69-1),"")</f>
@@ -8504,7 +8504,7 @@
         <v>516.37</v>
       </c>
       <c r="L70" s="5" t="n">
-        <v>578.4349999999999</v>
+        <v>560.260009765625</v>
       </c>
       <c r="M70" s="7">
         <f>IFERROR(IF(E70="Short",-1,1)*(IF(K70&lt;&gt;"",K70,L70)/J70-1),"")</f>
@@ -8575,7 +8575,7 @@
         <v>642.86</v>
       </c>
       <c r="L71" s="5" t="n">
-        <v>614.08</v>
+        <v>620.1900024414062</v>
       </c>
       <c r="M71" s="7">
         <f>IFERROR(IF(E71="Short",-1,1)*(IF(K71&lt;&gt;"",K71,L71)/J71-1),"")</f>
@@ -8646,7 +8646,7 @@
         <v>342.442857</v>
       </c>
       <c r="L72" s="5" t="n">
-        <v>351.9</v>
+        <v>342.3299865722656</v>
       </c>
       <c r="M72" s="7">
         <f>IFERROR(IF(E72="Short",-1,1)*(IF(K72&lt;&gt;"",K72,L72)/J72-1),"")</f>
@@ -8717,7 +8717,7 @@
         <v>168.09</v>
       </c>
       <c r="L73" s="5" t="n">
-        <v>166.98</v>
+        <v>168.1799926757812</v>
       </c>
       <c r="M73" s="7">
         <f>IFERROR(IF(E73="Short",-1,1)*(IF(K73&lt;&gt;"",K73,L73)/J73-1),"")</f>
@@ -8788,7 +8788,7 @@
         <v>240.841667</v>
       </c>
       <c r="L74" s="5" t="n">
-        <v>242.4</v>
+        <v>240.8899993896484</v>
       </c>
       <c r="M74" s="7">
         <f>IFERROR(IF(E74="Short",-1,1)*(IF(K74&lt;&gt;"",K74,L74)/J74-1),"")</f>
@@ -8859,7 +8859,7 @@
         <v>171.647334</v>
       </c>
       <c r="L75" s="5" t="n">
-        <v>172.76</v>
+        <v>171.5800018310547</v>
       </c>
       <c r="M75" s="7">
         <f>IFERROR(IF(E75="Short",-1,1)*(IF(K75&lt;&gt;"",K75,L75)/J75-1),"")</f>
@@ -8930,7 +8930,7 @@
         <v>243.820286</v>
       </c>
       <c r="L76" s="5" t="n">
-        <v>251.73</v>
+        <v>243.5700073242188</v>
       </c>
       <c r="M76" s="7">
         <f>IFERROR(IF(E76="Short",-1,1)*(IF(K76&lt;&gt;"",K76,L76)/J76-1),"")</f>
@@ -9001,7 +9001,7 @@
         <v>37.57</v>
       </c>
       <c r="L77" s="5" t="n">
-        <v>37.165</v>
+        <v>37.56000137329102</v>
       </c>
       <c r="M77" s="7">
         <f>IFERROR(IF(E77="Short",-1,1)*(IF(K77&lt;&gt;"",K77,L77)/J77-1),"")</f>
@@ -9072,7 +9072,7 @@
         <v>119.28</v>
       </c>
       <c r="L78" s="5" t="n">
-        <v>118.835</v>
+        <v>119.3199996948242</v>
       </c>
       <c r="M78" s="7">
         <f>IFERROR(IF(E78="Short",-1,1)*(IF(K78&lt;&gt;"",K78,L78)/J78-1),"")</f>
@@ -9143,7 +9143,7 @@
         <v>179.837143</v>
       </c>
       <c r="L79" s="5" t="n">
-        <v>182.08</v>
+        <v>179.9100036621094</v>
       </c>
       <c r="M79" s="7">
         <f>IFERROR(IF(E79="Short",-1,1)*(IF(K79&lt;&gt;"",K79,L79)/J79-1),"")</f>
@@ -9208,7 +9208,7 @@
       </c>
       <c r="K80" s="5" t="n"/>
       <c r="L80" s="5" t="n">
-        <v>773.08</v>
+        <v>769.6599731445312</v>
       </c>
       <c r="M80" s="7">
         <f>IFERROR(IF(E80="Short",-1,1)*(IF(K80&lt;&gt;"",K80,L80)/J80-1),"")</f>
@@ -9271,7 +9271,7 @@
       </c>
       <c r="K81" s="5" t="n"/>
       <c r="L81" s="5" t="n">
-        <v>551.54</v>
+        <v>531.3300170898438</v>
       </c>
       <c r="M81" s="7">
         <f>IFERROR(IF(E81="Short",-1,1)*(IF(K81&lt;&gt;"",K81,L81)/J81-1),"")</f>
@@ -9336,7 +9336,7 @@
       </c>
       <c r="K82" s="5" t="n"/>
       <c r="L82" s="5" t="n">
-        <v>62</v>
+        <v>62.52000045776367</v>
       </c>
       <c r="M82" s="7">
         <f>IFERROR(IF(E82="Short",-1,1)*(IF(K82&lt;&gt;"",K82,L82)/J82-1),"")</f>
@@ -9401,7 +9401,7 @@
       </c>
       <c r="K83" s="5" t="n"/>
       <c r="L83" s="5" t="n">
-        <v>35.83</v>
+        <v>35.09000015258789</v>
       </c>
       <c r="M83" s="7">
         <f>IFERROR(IF(E83="Short",-1,1)*(IF(K83&lt;&gt;"",K83,L83)/J83-1),"")</f>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="K84" s="5" t="n"/>
       <c r="L84" s="5" t="n">
-        <v>403.5</v>
+        <v>407.4599914550781</v>
       </c>
       <c r="M84" s="7">
         <f>IFERROR(IF(E84="Short",-1,1)*(IF(K84&lt;&gt;"",K84,L84)/J84-1),"")</f>
@@ -9531,7 +9531,7 @@
       </c>
       <c r="K85" s="5" t="n"/>
       <c r="L85" s="5" t="n">
-        <v>344.67</v>
+        <v>347.1000061035156</v>
       </c>
       <c r="M85" s="7">
         <f>IFERROR(IF(E85="Short",-1,1)*(IF(K85&lt;&gt;"",K85,L85)/J85-1),"")</f>
@@ -9596,7 +9596,7 @@
       </c>
       <c r="K86" s="5" t="n"/>
       <c r="L86" s="5" t="n">
-        <v>28.77</v>
+        <v>27.97999954223633</v>
       </c>
       <c r="M86" s="7">
         <f>IFERROR(IF(E86="Short",-1,1)*(IF(K86&lt;&gt;"",K86,L86)/J86-1),"")</f>
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K87" s="5" t="n"/>
       <c r="L87" s="5" t="n">
-        <v>52.38</v>
+        <v>52.27000045776367</v>
       </c>
       <c r="M87" s="7">
         <f>IFERROR(IF(E87="Short",-1,1)*(IF(K87&lt;&gt;"",K87,L87)/J87-1),"")</f>
@@ -9726,7 +9726,7 @@
       </c>
       <c r="K88" s="5" t="n"/>
       <c r="L88" s="5" t="n">
-        <v>118.65</v>
+        <v>118.3300018310547</v>
       </c>
       <c r="M88" s="7">
         <f>IFERROR(IF(E88="Short",-1,1)*(IF(K88&lt;&gt;"",K88,L88)/J88-1),"")</f>
@@ -9791,7 +9791,7 @@
       </c>
       <c r="K89" s="5" t="n"/>
       <c r="L89" s="5" t="n">
-        <v>253.86</v>
+        <v>240.8500061035156</v>
       </c>
       <c r="M89" s="7">
         <f>IFERROR(IF(E89="Short",-1,1)*(IF(K89&lt;&gt;"",K89,L89)/J89-1),"")</f>
@@ -9856,7 +9856,7 @@
       </c>
       <c r="K90" s="5" t="n"/>
       <c r="L90" s="5" t="n">
-        <v>33.51</v>
+        <v>34.0099983215332</v>
       </c>
       <c r="M90" s="7">
         <f>IFERROR(IF(E90="Short",-1,1)*(IF(K90&lt;&gt;"",K90,L90)/J90-1),"")</f>

</xml_diff>